<commit_message>
VAR formula on excel fixed
</commit_message>
<xml_diff>
--- a/sample/VAR-REPORT.xlsx
+++ b/sample/VAR-REPORT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Miks\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0B6AEAD2-F355-4173-9DC8-4CC1C19D8754}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F466E4D-3CD3-4DFC-90AE-3F09EBB2C565}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{39334F03-1232-460D-B301-DE63E4B3EB5C}"/>
   </bookViews>
@@ -1115,6 +1115,54 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" wrapText="1"/>
       <protection locked="0"/>
@@ -1135,6 +1183,10 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -1159,10 +1211,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -1217,54 +1265,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -1662,107 +1662,107 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:18" ht="15">
-      <c r="B1" s="93" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="93"/>
-      <c r="D1" s="93"/>
-      <c r="E1" s="93"/>
-      <c r="F1" s="93"/>
-      <c r="G1" s="93"/>
-      <c r="H1" s="93"/>
-      <c r="I1" s="93"/>
-      <c r="J1" s="93"/>
-      <c r="K1" s="93"/>
-      <c r="L1" s="93"/>
-      <c r="M1" s="93"/>
-      <c r="N1" s="93"/>
-      <c r="O1" s="93"/>
-      <c r="P1" s="93"/>
-      <c r="Q1" s="93"/>
-      <c r="R1" s="93"/>
+      <c r="B1" s="70" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="70"/>
+      <c r="D1" s="70"/>
+      <c r="E1" s="70"/>
+      <c r="F1" s="70"/>
+      <c r="G1" s="70"/>
+      <c r="H1" s="70"/>
+      <c r="I1" s="70"/>
+      <c r="J1" s="70"/>
+      <c r="K1" s="70"/>
+      <c r="L1" s="70"/>
+      <c r="M1" s="70"/>
+      <c r="N1" s="70"/>
+      <c r="O1" s="70"/>
+      <c r="P1" s="70"/>
+      <c r="Q1" s="70"/>
+      <c r="R1" s="70"/>
     </row>
     <row r="2" spans="2:18" ht="15">
-      <c r="B2" s="93" t="s">
+      <c r="B2" s="70" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="93"/>
-      <c r="D2" s="93"/>
-      <c r="E2" s="93"/>
-      <c r="F2" s="93"/>
-      <c r="G2" s="93"/>
-      <c r="H2" s="93"/>
-      <c r="I2" s="93"/>
-      <c r="J2" s="93"/>
-      <c r="K2" s="93"/>
-      <c r="L2" s="93"/>
-      <c r="M2" s="93"/>
-      <c r="N2" s="93"/>
-      <c r="O2" s="93"/>
-      <c r="P2" s="93"/>
-      <c r="Q2" s="93"/>
-      <c r="R2" s="93"/>
+      <c r="C2" s="70"/>
+      <c r="D2" s="70"/>
+      <c r="E2" s="70"/>
+      <c r="F2" s="70"/>
+      <c r="G2" s="70"/>
+      <c r="H2" s="70"/>
+      <c r="I2" s="70"/>
+      <c r="J2" s="70"/>
+      <c r="K2" s="70"/>
+      <c r="L2" s="70"/>
+      <c r="M2" s="70"/>
+      <c r="N2" s="70"/>
+      <c r="O2" s="70"/>
+      <c r="P2" s="70"/>
+      <c r="Q2" s="70"/>
+      <c r="R2" s="70"/>
     </row>
     <row r="3" spans="2:18">
-      <c r="B3" s="94" t="s">
+      <c r="B3" s="71" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="94"/>
-      <c r="D3" s="94"/>
-      <c r="E3" s="94"/>
-      <c r="F3" s="94"/>
-      <c r="G3" s="94"/>
-      <c r="H3" s="94"/>
-      <c r="I3" s="94"/>
-      <c r="J3" s="94"/>
-      <c r="K3" s="94"/>
-      <c r="L3" s="94"/>
-      <c r="M3" s="94"/>
-      <c r="N3" s="94"/>
-      <c r="O3" s="94"/>
-      <c r="P3" s="94"/>
-      <c r="Q3" s="94"/>
-      <c r="R3" s="94"/>
+      <c r="C3" s="71"/>
+      <c r="D3" s="71"/>
+      <c r="E3" s="71"/>
+      <c r="F3" s="71"/>
+      <c r="G3" s="71"/>
+      <c r="H3" s="71"/>
+      <c r="I3" s="71"/>
+      <c r="J3" s="71"/>
+      <c r="K3" s="71"/>
+      <c r="L3" s="71"/>
+      <c r="M3" s="71"/>
+      <c r="N3" s="71"/>
+      <c r="O3" s="71"/>
+      <c r="P3" s="71"/>
+      <c r="Q3" s="71"/>
+      <c r="R3" s="71"/>
     </row>
     <row r="4" spans="2:18">
-      <c r="B4" s="95" t="s">
+      <c r="B4" s="72" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="95"/>
-      <c r="D4" s="95"/>
-      <c r="E4" s="95"/>
-      <c r="F4" s="95"/>
-      <c r="G4" s="95"/>
-      <c r="H4" s="95"/>
-      <c r="I4" s="95"/>
-      <c r="J4" s="95"/>
-      <c r="K4" s="95"/>
-      <c r="L4" s="95"/>
-      <c r="M4" s="95"/>
-      <c r="N4" s="95"/>
-      <c r="O4" s="95"/>
-      <c r="P4" s="95"/>
-      <c r="Q4" s="95"/>
-      <c r="R4" s="95"/>
+      <c r="C4" s="72"/>
+      <c r="D4" s="72"/>
+      <c r="E4" s="72"/>
+      <c r="F4" s="72"/>
+      <c r="G4" s="72"/>
+      <c r="H4" s="72"/>
+      <c r="I4" s="72"/>
+      <c r="J4" s="72"/>
+      <c r="K4" s="72"/>
+      <c r="L4" s="72"/>
+      <c r="M4" s="72"/>
+      <c r="N4" s="72"/>
+      <c r="O4" s="72"/>
+      <c r="P4" s="72"/>
+      <c r="Q4" s="72"/>
+      <c r="R4" s="72"/>
     </row>
     <row r="5" spans="2:18" ht="15">
-      <c r="B5" s="96"/>
-      <c r="C5" s="96"/>
-      <c r="D5" s="96"/>
-      <c r="E5" s="96"/>
-      <c r="F5" s="96"/>
-      <c r="G5" s="96"/>
-      <c r="H5" s="96"/>
-      <c r="I5" s="96"/>
-      <c r="J5" s="96"/>
-      <c r="K5" s="96"/>
-      <c r="L5" s="96"/>
-      <c r="M5" s="96"/>
-      <c r="N5" s="96"/>
-      <c r="O5" s="96"/>
-      <c r="P5" s="96"/>
-      <c r="Q5" s="96"/>
-      <c r="R5" s="96"/>
+      <c r="B5" s="73"/>
+      <c r="C5" s="73"/>
+      <c r="D5" s="73"/>
+      <c r="E5" s="73"/>
+      <c r="F5" s="73"/>
+      <c r="G5" s="73"/>
+      <c r="H5" s="73"/>
+      <c r="I5" s="73"/>
+      <c r="J5" s="73"/>
+      <c r="K5" s="73"/>
+      <c r="L5" s="73"/>
+      <c r="M5" s="73"/>
+      <c r="N5" s="73"/>
+      <c r="O5" s="73"/>
+      <c r="P5" s="73"/>
+      <c r="Q5" s="73"/>
+      <c r="R5" s="73"/>
     </row>
     <row r="6" spans="2:18" ht="15">
       <c r="B6" s="2" t="s">
@@ -1891,85 +1891,85 @@
       <c r="R11" s="9"/>
     </row>
     <row r="12" spans="2:18" ht="16.5" customHeight="1">
-      <c r="B12" s="97" t="s">
+      <c r="B12" s="62" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="98"/>
-      <c r="D12" s="63" t="s">
+      <c r="C12" s="63"/>
+      <c r="D12" s="76" t="s">
         <v>10</v>
       </c>
-      <c r="E12" s="64"/>
-      <c r="F12" s="64"/>
-      <c r="G12" s="64"/>
-      <c r="H12" s="64"/>
-      <c r="I12" s="64"/>
-      <c r="J12" s="64"/>
-      <c r="K12" s="64"/>
-      <c r="L12" s="64"/>
-      <c r="M12" s="64"/>
-      <c r="N12" s="64"/>
-      <c r="O12" s="65"/>
-      <c r="P12" s="78" t="s">
+      <c r="E12" s="77"/>
+      <c r="F12" s="77"/>
+      <c r="G12" s="77"/>
+      <c r="H12" s="77"/>
+      <c r="I12" s="77"/>
+      <c r="J12" s="77"/>
+      <c r="K12" s="77"/>
+      <c r="L12" s="77"/>
+      <c r="M12" s="77"/>
+      <c r="N12" s="77"/>
+      <c r="O12" s="78"/>
+      <c r="P12" s="91" t="s">
         <v>11</v>
       </c>
-      <c r="Q12" s="79"/>
-      <c r="R12" s="80"/>
+      <c r="Q12" s="92"/>
+      <c r="R12" s="93"/>
     </row>
     <row r="13" spans="2:18" ht="15" customHeight="1">
-      <c r="B13" s="66" t="s">
+      <c r="B13" s="80" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="69" t="s">
+      <c r="C13" s="83" t="s">
         <v>13</v>
       </c>
-      <c r="D13" s="85" t="s">
+      <c r="D13" s="98" t="s">
         <v>14</v>
       </c>
-      <c r="E13" s="86"/>
-      <c r="F13" s="86"/>
-      <c r="G13" s="86"/>
-      <c r="H13" s="86"/>
-      <c r="I13" s="86"/>
-      <c r="J13" s="86"/>
-      <c r="K13" s="86"/>
-      <c r="L13" s="86"/>
-      <c r="M13" s="66" t="s">
+      <c r="E13" s="99"/>
+      <c r="F13" s="99"/>
+      <c r="G13" s="99"/>
+      <c r="H13" s="99"/>
+      <c r="I13" s="99"/>
+      <c r="J13" s="99"/>
+      <c r="K13" s="99"/>
+      <c r="L13" s="99"/>
+      <c r="M13" s="80" t="s">
         <v>15</v>
       </c>
-      <c r="N13" s="73"/>
-      <c r="O13" s="74"/>
-      <c r="P13" s="67"/>
-      <c r="Q13" s="81"/>
-      <c r="R13" s="82"/>
+      <c r="N13" s="86"/>
+      <c r="O13" s="87"/>
+      <c r="P13" s="81"/>
+      <c r="Q13" s="94"/>
+      <c r="R13" s="95"/>
     </row>
     <row r="14" spans="2:18" ht="28.5" customHeight="1" thickBot="1">
-      <c r="B14" s="67"/>
-      <c r="C14" s="70"/>
-      <c r="D14" s="87" t="s">
+      <c r="B14" s="81"/>
+      <c r="C14" s="84"/>
+      <c r="D14" s="64" t="s">
         <v>27</v>
       </c>
-      <c r="E14" s="88"/>
-      <c r="F14" s="89"/>
-      <c r="G14" s="87" t="s">
+      <c r="E14" s="65"/>
+      <c r="F14" s="66"/>
+      <c r="G14" s="64" t="s">
         <v>28</v>
       </c>
-      <c r="H14" s="88"/>
-      <c r="I14" s="89"/>
-      <c r="J14" s="87" t="s">
+      <c r="H14" s="65"/>
+      <c r="I14" s="66"/>
+      <c r="J14" s="64" t="s">
         <v>29</v>
       </c>
-      <c r="K14" s="88"/>
-      <c r="L14" s="89"/>
-      <c r="M14" s="75"/>
-      <c r="N14" s="76"/>
-      <c r="O14" s="77"/>
-      <c r="P14" s="68"/>
-      <c r="Q14" s="83"/>
-      <c r="R14" s="84"/>
+      <c r="K14" s="65"/>
+      <c r="L14" s="66"/>
+      <c r="M14" s="88"/>
+      <c r="N14" s="89"/>
+      <c r="O14" s="90"/>
+      <c r="P14" s="82"/>
+      <c r="Q14" s="96"/>
+      <c r="R14" s="97"/>
     </row>
     <row r="15" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
-      <c r="B15" s="68"/>
-      <c r="C15" s="71"/>
+      <c r="B15" s="82"/>
+      <c r="C15" s="85"/>
       <c r="D15" s="10" t="s">
         <v>16</v>
       </c>
@@ -2016,31 +2016,27 @@
       <c r="D16" s="16"/>
       <c r="E16" s="17"/>
       <c r="F16" s="18">
-        <f t="shared" ref="F16:F45" si="0">D16+E16</f>
         <v>0</v>
       </c>
       <c r="G16" s="19"/>
       <c r="H16" s="48"/>
       <c r="I16" s="49">
-        <f t="shared" ref="I16:I56" si="1">G16+H16</f>
         <v>0</v>
       </c>
       <c r="J16" s="19"/>
       <c r="K16" s="20"/>
       <c r="L16" s="47">
-        <f t="shared" ref="L16:L45" si="2">J16+K16</f>
         <v>0</v>
       </c>
       <c r="M16" s="19"/>
       <c r="N16" s="48"/>
       <c r="O16" s="49">
-        <f t="shared" ref="O16:O45" si="3">M16+N16</f>
         <v>0</v>
       </c>
       <c r="P16" s="50"/>
       <c r="Q16" s="50"/>
       <c r="R16" s="50">
-        <f t="shared" ref="R16:R56" si="4">F16+L16+O16</f>
+        <f>F16+I16+S16+L16+O16</f>
         <v>0</v>
       </c>
     </row>
@@ -2050,31 +2046,31 @@
       <c r="D17" s="23"/>
       <c r="E17" s="24"/>
       <c r="F17" s="18">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="F16:F45" si="0">D17+E17</f>
         <v>0</v>
       </c>
       <c r="G17" s="25"/>
       <c r="H17" s="51"/>
       <c r="I17" s="49">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="I16:I56" si="1">G17+H17</f>
         <v>0</v>
       </c>
       <c r="J17" s="25"/>
       <c r="K17" s="26"/>
       <c r="L17" s="47">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="L16:L45" si="2">J17+K17</f>
         <v>0</v>
       </c>
       <c r="M17" s="25"/>
       <c r="N17" s="51"/>
       <c r="O17" s="49">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="O16:O45" si="3">M17+N17</f>
         <v>0</v>
       </c>
       <c r="P17" s="52"/>
       <c r="Q17" s="52"/>
       <c r="R17" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="R17:R57" si="4">F17+I17+S17+L17+O17</f>
         <v>0</v>
       </c>
     </row>
@@ -3405,10 +3401,10 @@
       </c>
     </row>
     <row r="57" spans="2:18" ht="33.75" customHeight="1" thickBot="1">
-      <c r="B57" s="61" t="s">
+      <c r="B57" s="74" t="s">
         <v>20</v>
       </c>
-      <c r="C57" s="62"/>
+      <c r="C57" s="75"/>
       <c r="D57" s="41">
         <f>SUM(D16:D56)</f>
         <v>0</v>
@@ -3461,8 +3457,8 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="R57" s="41">
-        <f t="shared" si="8"/>
+      <c r="R57" s="50">
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -3494,55 +3490,55 @@
       <c r="F59" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="N59" s="90" t="s">
+      <c r="N59" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="O59" s="90"/>
+      <c r="O59" s="67"/>
     </row>
     <row r="60" spans="2:18" ht="21" customHeight="1"/>
     <row r="61" spans="2:18" ht="21" customHeight="1">
       <c r="B61" s="43" t="s">
         <v>32</v>
       </c>
-      <c r="G61" s="91" t="s">
+      <c r="G61" s="68" t="s">
         <v>33</v>
       </c>
-      <c r="H61" s="91"/>
-      <c r="I61" s="91"/>
-      <c r="J61" s="91"/>
-      <c r="N61" s="92" t="s">
+      <c r="H61" s="68"/>
+      <c r="I61" s="68"/>
+      <c r="J61" s="68"/>
+      <c r="N61" s="69" t="s">
         <v>25</v>
       </c>
-      <c r="O61" s="92"/>
-      <c r="P61" s="92"/>
-      <c r="Q61" s="92"/>
+      <c r="O61" s="69"/>
+      <c r="P61" s="69"/>
+      <c r="Q61" s="69"/>
     </row>
     <row r="62" spans="2:18" ht="21" customHeight="1">
       <c r="B62" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="G62" s="72" t="s">
+      <c r="G62" s="79" t="s">
         <v>31</v>
       </c>
-      <c r="H62" s="72"/>
-      <c r="I62" s="72"/>
-      <c r="J62" s="72"/>
-      <c r="N62" s="72" t="s">
+      <c r="H62" s="79"/>
+      <c r="I62" s="79"/>
+      <c r="J62" s="79"/>
+      <c r="N62" s="79" t="s">
         <v>35</v>
       </c>
-      <c r="O62" s="72"/>
-      <c r="P62" s="72"/>
-      <c r="Q62" s="72"/>
+      <c r="O62" s="79"/>
+      <c r="P62" s="79"/>
+      <c r="Q62" s="79"/>
     </row>
     <row r="63" spans="2:18" ht="21" customHeight="1">
-      <c r="G63" s="99"/>
-      <c r="H63" s="99"/>
-      <c r="I63" s="99"/>
-      <c r="J63" s="99"/>
-      <c r="N63" s="72"/>
-      <c r="O63" s="72"/>
-      <c r="P63" s="72"/>
-      <c r="Q63" s="72"/>
+      <c r="G63" s="61"/>
+      <c r="H63" s="61"/>
+      <c r="I63" s="61"/>
+      <c r="J63" s="61"/>
+      <c r="N63" s="79"/>
+      <c r="O63" s="79"/>
+      <c r="P63" s="79"/>
+      <c r="Q63" s="79"/>
     </row>
     <row r="64" spans="2:18" ht="21" customHeight="1">
       <c r="B64" s="1" t="s">
@@ -3575,19 +3571,6 @@
     <row r="86" ht="21" customHeight="1"/>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="J14:L14"/>
-    <mergeCell ref="G14:I14"/>
-    <mergeCell ref="N59:O59"/>
-    <mergeCell ref="G61:J61"/>
-    <mergeCell ref="N61:Q61"/>
-    <mergeCell ref="B1:R1"/>
-    <mergeCell ref="B2:R2"/>
-    <mergeCell ref="B3:R3"/>
-    <mergeCell ref="B4:R4"/>
-    <mergeCell ref="B5:R5"/>
-    <mergeCell ref="B57:C57"/>
-    <mergeCell ref="D12:O12"/>
     <mergeCell ref="G62:J62"/>
     <mergeCell ref="B13:B15"/>
     <mergeCell ref="C13:C15"/>
@@ -3596,6 +3579,19 @@
     <mergeCell ref="P12:R14"/>
     <mergeCell ref="D13:L13"/>
     <mergeCell ref="D14:F14"/>
+    <mergeCell ref="B1:R1"/>
+    <mergeCell ref="B2:R2"/>
+    <mergeCell ref="B3:R3"/>
+    <mergeCell ref="B4:R4"/>
+    <mergeCell ref="B5:R5"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="J14:L14"/>
+    <mergeCell ref="G14:I14"/>
+    <mergeCell ref="N59:O59"/>
+    <mergeCell ref="G61:J61"/>
+    <mergeCell ref="N61:Q61"/>
+    <mergeCell ref="B57:C57"/>
+    <mergeCell ref="D12:O12"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B4" r:id="rId1" xr:uid="{5EAE8D1D-5A31-4631-AC47-0FB40220C481}"/>

</xml_diff>

<commit_message>
Both apply to every sheet (VAR, DAE daily, DAE monthly) — any formula cell where ExcelJS drops result: 0 will now show a right-aligned "0".
</commit_message>
<xml_diff>
--- a/sample/VAR-REPORT.xlsx
+++ b/sample/VAR-REPORT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Miks\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F466E4D-3CD3-4DFC-90AE-3F09EBB2C565}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04A4C52E-30AA-4CBF-A3E0-5E38AB1289A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{39334F03-1232-460D-B301-DE63E4B3EB5C}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="36">
   <si>
     <t>Republic of the Philippines</t>
   </si>
@@ -261,7 +261,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="51">
+  <borders count="46">
     <border>
       <left/>
       <right/>
@@ -696,58 +696,6 @@
       <left style="medium">
         <color indexed="64"/>
       </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -854,17 +802,6 @@
         <color indexed="64"/>
       </top>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -895,7 +832,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="100">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0"/>
@@ -1084,9 +1021,6 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="2" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="3" fontId="1" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -1095,23 +1029,14 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="2" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="2" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="2" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="4" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="3" fontId="1" fillId="4" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -1119,6 +1044,102 @@
       <alignment vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -1127,18 +1148,6 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -1151,120 +1160,24 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -1662,107 +1575,107 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:18" ht="15">
-      <c r="B1" s="70" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="70"/>
-      <c r="D1" s="70"/>
-      <c r="E1" s="70"/>
-      <c r="F1" s="70"/>
-      <c r="G1" s="70"/>
-      <c r="H1" s="70"/>
-      <c r="I1" s="70"/>
-      <c r="J1" s="70"/>
-      <c r="K1" s="70"/>
-      <c r="L1" s="70"/>
-      <c r="M1" s="70"/>
-      <c r="N1" s="70"/>
-      <c r="O1" s="70"/>
-      <c r="P1" s="70"/>
-      <c r="Q1" s="70"/>
-      <c r="R1" s="70"/>
+      <c r="B1" s="58" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="58"/>
+      <c r="D1" s="58"/>
+      <c r="E1" s="58"/>
+      <c r="F1" s="58"/>
+      <c r="G1" s="58"/>
+      <c r="H1" s="58"/>
+      <c r="I1" s="58"/>
+      <c r="J1" s="58"/>
+      <c r="K1" s="58"/>
+      <c r="L1" s="58"/>
+      <c r="M1" s="58"/>
+      <c r="N1" s="58"/>
+      <c r="O1" s="58"/>
+      <c r="P1" s="58"/>
+      <c r="Q1" s="58"/>
+      <c r="R1" s="58"/>
     </row>
     <row r="2" spans="2:18" ht="15">
-      <c r="B2" s="70" t="s">
+      <c r="B2" s="58" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
-      <c r="K2" s="70"/>
-      <c r="L2" s="70"/>
-      <c r="M2" s="70"/>
-      <c r="N2" s="70"/>
-      <c r="O2" s="70"/>
-      <c r="P2" s="70"/>
-      <c r="Q2" s="70"/>
-      <c r="R2" s="70"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
+      <c r="H2" s="58"/>
+      <c r="I2" s="58"/>
+      <c r="J2" s="58"/>
+      <c r="K2" s="58"/>
+      <c r="L2" s="58"/>
+      <c r="M2" s="58"/>
+      <c r="N2" s="58"/>
+      <c r="O2" s="58"/>
+      <c r="P2" s="58"/>
+      <c r="Q2" s="58"/>
+      <c r="R2" s="58"/>
     </row>
     <row r="3" spans="2:18">
-      <c r="B3" s="71" t="s">
+      <c r="B3" s="59" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="71"/>
-      <c r="D3" s="71"/>
-      <c r="E3" s="71"/>
-      <c r="F3" s="71"/>
-      <c r="G3" s="71"/>
-      <c r="H3" s="71"/>
-      <c r="I3" s="71"/>
-      <c r="J3" s="71"/>
-      <c r="K3" s="71"/>
-      <c r="L3" s="71"/>
-      <c r="M3" s="71"/>
-      <c r="N3" s="71"/>
-      <c r="O3" s="71"/>
-      <c r="P3" s="71"/>
-      <c r="Q3" s="71"/>
-      <c r="R3" s="71"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="59"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="59"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="59"/>
+      <c r="L3" s="59"/>
+      <c r="M3" s="59"/>
+      <c r="N3" s="59"/>
+      <c r="O3" s="59"/>
+      <c r="P3" s="59"/>
+      <c r="Q3" s="59"/>
+      <c r="R3" s="59"/>
     </row>
     <row r="4" spans="2:18">
-      <c r="B4" s="72" t="s">
+      <c r="B4" s="60" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="72"/>
-      <c r="D4" s="72"/>
-      <c r="E4" s="72"/>
-      <c r="F4" s="72"/>
-      <c r="G4" s="72"/>
-      <c r="H4" s="72"/>
-      <c r="I4" s="72"/>
-      <c r="J4" s="72"/>
-      <c r="K4" s="72"/>
-      <c r="L4" s="72"/>
-      <c r="M4" s="72"/>
-      <c r="N4" s="72"/>
-      <c r="O4" s="72"/>
-      <c r="P4" s="72"/>
-      <c r="Q4" s="72"/>
-      <c r="R4" s="72"/>
+      <c r="C4" s="60"/>
+      <c r="D4" s="60"/>
+      <c r="E4" s="60"/>
+      <c r="F4" s="60"/>
+      <c r="G4" s="60"/>
+      <c r="H4" s="60"/>
+      <c r="I4" s="60"/>
+      <c r="J4" s="60"/>
+      <c r="K4" s="60"/>
+      <c r="L4" s="60"/>
+      <c r="M4" s="60"/>
+      <c r="N4" s="60"/>
+      <c r="O4" s="60"/>
+      <c r="P4" s="60"/>
+      <c r="Q4" s="60"/>
+      <c r="R4" s="60"/>
     </row>
     <row r="5" spans="2:18" ht="15">
-      <c r="B5" s="73"/>
-      <c r="C5" s="73"/>
-      <c r="D5" s="73"/>
-      <c r="E5" s="73"/>
-      <c r="F5" s="73"/>
-      <c r="G5" s="73"/>
-      <c r="H5" s="73"/>
-      <c r="I5" s="73"/>
-      <c r="J5" s="73"/>
-      <c r="K5" s="73"/>
-      <c r="L5" s="73"/>
-      <c r="M5" s="73"/>
-      <c r="N5" s="73"/>
-      <c r="O5" s="73"/>
-      <c r="P5" s="73"/>
-      <c r="Q5" s="73"/>
-      <c r="R5" s="73"/>
+      <c r="B5" s="61"/>
+      <c r="C5" s="61"/>
+      <c r="D5" s="61"/>
+      <c r="E5" s="61"/>
+      <c r="F5" s="61"/>
+      <c r="G5" s="61"/>
+      <c r="H5" s="61"/>
+      <c r="I5" s="61"/>
+      <c r="J5" s="61"/>
+      <c r="K5" s="61"/>
+      <c r="L5" s="61"/>
+      <c r="M5" s="61"/>
+      <c r="N5" s="61"/>
+      <c r="O5" s="61"/>
+      <c r="P5" s="61"/>
+      <c r="Q5" s="61"/>
+      <c r="R5" s="61"/>
     </row>
     <row r="6" spans="2:18" ht="15">
       <c r="B6" s="2" t="s">
@@ -1891,85 +1804,85 @@
       <c r="R11" s="9"/>
     </row>
     <row r="12" spans="2:18" ht="16.5" customHeight="1">
-      <c r="B12" s="62" t="s">
+      <c r="B12" s="83" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="63"/>
-      <c r="D12" s="76" t="s">
+      <c r="C12" s="84"/>
+      <c r="D12" s="90" t="s">
         <v>10</v>
       </c>
-      <c r="E12" s="77"/>
-      <c r="F12" s="77"/>
-      <c r="G12" s="77"/>
-      <c r="H12" s="77"/>
-      <c r="I12" s="77"/>
-      <c r="J12" s="77"/>
-      <c r="K12" s="77"/>
-      <c r="L12" s="77"/>
-      <c r="M12" s="77"/>
-      <c r="N12" s="77"/>
-      <c r="O12" s="78"/>
-      <c r="P12" s="91" t="s">
+      <c r="E12" s="91"/>
+      <c r="F12" s="91"/>
+      <c r="G12" s="91"/>
+      <c r="H12" s="91"/>
+      <c r="I12" s="91"/>
+      <c r="J12" s="91"/>
+      <c r="K12" s="91"/>
+      <c r="L12" s="91"/>
+      <c r="M12" s="91"/>
+      <c r="N12" s="91"/>
+      <c r="O12" s="92"/>
+      <c r="P12" s="71" t="s">
         <v>11</v>
       </c>
-      <c r="Q12" s="92"/>
-      <c r="R12" s="93"/>
+      <c r="Q12" s="72"/>
+      <c r="R12" s="73"/>
     </row>
     <row r="13" spans="2:18" ht="15" customHeight="1">
-      <c r="B13" s="80" t="s">
+      <c r="B13" s="63" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="83" t="s">
+      <c r="C13" s="66" t="s">
         <v>13</v>
       </c>
-      <c r="D13" s="98" t="s">
+      <c r="D13" s="78" t="s">
         <v>14</v>
       </c>
-      <c r="E13" s="99"/>
-      <c r="F13" s="99"/>
-      <c r="G13" s="99"/>
-      <c r="H13" s="99"/>
-      <c r="I13" s="99"/>
-      <c r="J13" s="99"/>
-      <c r="K13" s="99"/>
-      <c r="L13" s="99"/>
-      <c r="M13" s="80" t="s">
+      <c r="E13" s="79"/>
+      <c r="F13" s="79"/>
+      <c r="G13" s="79"/>
+      <c r="H13" s="79"/>
+      <c r="I13" s="79"/>
+      <c r="J13" s="79"/>
+      <c r="K13" s="79"/>
+      <c r="L13" s="79"/>
+      <c r="M13" s="63" t="s">
         <v>15</v>
       </c>
-      <c r="N13" s="86"/>
-      <c r="O13" s="87"/>
-      <c r="P13" s="81"/>
-      <c r="Q13" s="94"/>
-      <c r="R13" s="95"/>
+      <c r="N13" s="69"/>
+      <c r="O13" s="70"/>
+      <c r="P13" s="64"/>
+      <c r="Q13" s="74"/>
+      <c r="R13" s="75"/>
     </row>
     <row r="14" spans="2:18" ht="28.5" customHeight="1" thickBot="1">
-      <c r="B14" s="81"/>
-      <c r="C14" s="84"/>
-      <c r="D14" s="64" t="s">
+      <c r="B14" s="64"/>
+      <c r="C14" s="67"/>
+      <c r="D14" s="80" t="s">
         <v>27</v>
       </c>
-      <c r="E14" s="65"/>
-      <c r="F14" s="66"/>
-      <c r="G14" s="64" t="s">
+      <c r="E14" s="81"/>
+      <c r="F14" s="82"/>
+      <c r="G14" s="80" t="s">
         <v>28</v>
       </c>
-      <c r="H14" s="65"/>
-      <c r="I14" s="66"/>
-      <c r="J14" s="64" t="s">
+      <c r="H14" s="81"/>
+      <c r="I14" s="82"/>
+      <c r="J14" s="80" t="s">
         <v>29</v>
       </c>
-      <c r="K14" s="65"/>
-      <c r="L14" s="66"/>
-      <c r="M14" s="88"/>
-      <c r="N14" s="89"/>
-      <c r="O14" s="90"/>
-      <c r="P14" s="82"/>
-      <c r="Q14" s="96"/>
-      <c r="R14" s="97"/>
+      <c r="K14" s="81"/>
+      <c r="L14" s="82"/>
+      <c r="M14" s="65"/>
+      <c r="N14" s="76"/>
+      <c r="O14" s="77"/>
+      <c r="P14" s="65"/>
+      <c r="Q14" s="76"/>
+      <c r="R14" s="77"/>
     </row>
     <row r="15" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
-      <c r="B15" s="82"/>
-      <c r="C15" s="85"/>
+      <c r="B15" s="65"/>
+      <c r="C15" s="68"/>
       <c r="D15" s="10" t="s">
         <v>16</v>
       </c>
@@ -1979,9 +1892,15 @@
       <c r="F15" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="G15" s="60"/>
-      <c r="H15" s="60"/>
-      <c r="I15" s="60"/>
+      <c r="G15" s="56" t="s">
+        <v>16</v>
+      </c>
+      <c r="H15" s="56" t="s">
+        <v>17</v>
+      </c>
+      <c r="I15" s="56" t="s">
+        <v>18</v>
+      </c>
       <c r="J15" s="10" t="s">
         <v>16</v>
       </c>
@@ -2016,27 +1935,37 @@
       <c r="D16" s="16"/>
       <c r="E16" s="17"/>
       <c r="F16" s="18">
+        <f t="shared" ref="F16:F45" si="0">D16+E16</f>
         <v>0</v>
       </c>
       <c r="G16" s="19"/>
       <c r="H16" s="48"/>
       <c r="I16" s="49">
+        <f t="shared" ref="I16:I56" si="1">G16+H16</f>
         <v>0</v>
       </c>
       <c r="J16" s="19"/>
       <c r="K16" s="20"/>
       <c r="L16" s="47">
+        <f t="shared" ref="L16:L45" si="2">J16+K16</f>
         <v>0</v>
       </c>
       <c r="M16" s="19"/>
       <c r="N16" s="48"/>
       <c r="O16" s="49">
-        <v>0</v>
-      </c>
-      <c r="P16" s="50"/>
-      <c r="Q16" s="50"/>
+        <f t="shared" ref="O16:O45" si="3">M16+N16</f>
+        <v>0</v>
+      </c>
+      <c r="P16" s="50">
+        <f>D16+G16+J16+M16</f>
+        <v>0</v>
+      </c>
+      <c r="Q16" s="50">
+        <f>E16+H16+K16+N16</f>
+        <v>0</v>
+      </c>
       <c r="R16" s="50">
-        <f>F16+I16+S16+L16+O16</f>
+        <f>F16+I16+L16+O16</f>
         <v>0</v>
       </c>
     </row>
@@ -2046,31 +1975,37 @@
       <c r="D17" s="23"/>
       <c r="E17" s="24"/>
       <c r="F17" s="18">
-        <f t="shared" ref="F16:F45" si="0">D17+E17</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="G17" s="25"/>
       <c r="H17" s="51"/>
       <c r="I17" s="49">
-        <f t="shared" ref="I16:I56" si="1">G17+H17</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J17" s="25"/>
       <c r="K17" s="26"/>
       <c r="L17" s="47">
-        <f t="shared" ref="L16:L45" si="2">J17+K17</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M17" s="25"/>
       <c r="N17" s="51"/>
       <c r="O17" s="49">
-        <f t="shared" ref="O16:O45" si="3">M17+N17</f>
-        <v>0</v>
-      </c>
-      <c r="P17" s="52"/>
-      <c r="Q17" s="52"/>
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="P17" s="50">
+        <f t="shared" ref="P17:P56" si="4">D17+G17+J17+M17</f>
+        <v>0</v>
+      </c>
+      <c r="Q17" s="50">
+        <f t="shared" ref="Q17:Q56" si="5">E17+H17+K17+N17</f>
+        <v>0</v>
+      </c>
       <c r="R17" s="50">
-        <f t="shared" ref="R17:R57" si="4">F17+I17+S17+L17+O17</f>
+        <f t="shared" ref="R17:R57" si="6">F17+I17+L17+O17</f>
         <v>0</v>
       </c>
     </row>
@@ -2101,10 +2036,16 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P18" s="52"/>
-      <c r="Q18" s="52"/>
+      <c r="P18" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q18" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R18" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -2118,7 +2059,7 @@
         <v>0</v>
       </c>
       <c r="G19" s="29"/>
-      <c r="H19" s="53"/>
+      <c r="H19" s="52"/>
       <c r="I19" s="49">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -2130,15 +2071,21 @@
         <v>0</v>
       </c>
       <c r="M19" s="29"/>
-      <c r="N19" s="53"/>
+      <c r="N19" s="52"/>
       <c r="O19" s="49">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P19" s="52"/>
-      <c r="Q19" s="52"/>
+      <c r="P19" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q19" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R19" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -2152,7 +2099,7 @@
         <v>0</v>
       </c>
       <c r="G20" s="29"/>
-      <c r="H20" s="53"/>
+      <c r="H20" s="52"/>
       <c r="I20" s="49">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -2164,15 +2111,21 @@
         <v>0</v>
       </c>
       <c r="M20" s="29"/>
-      <c r="N20" s="53"/>
+      <c r="N20" s="52"/>
       <c r="O20" s="49">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P20" s="52"/>
-      <c r="Q20" s="52"/>
+      <c r="P20" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q20" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R20" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -2186,7 +2139,7 @@
         <v>0</v>
       </c>
       <c r="G21" s="29"/>
-      <c r="H21" s="53"/>
+      <c r="H21" s="52"/>
       <c r="I21" s="49">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -2198,15 +2151,21 @@
         <v>0</v>
       </c>
       <c r="M21" s="29"/>
-      <c r="N21" s="53"/>
+      <c r="N21" s="52"/>
       <c r="O21" s="49">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P21" s="52"/>
-      <c r="Q21" s="52"/>
+      <c r="P21" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q21" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R21" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -2220,7 +2179,7 @@
         <v>0</v>
       </c>
       <c r="G22" s="29"/>
-      <c r="H22" s="53"/>
+      <c r="H22" s="52"/>
       <c r="I22" s="49">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -2232,15 +2191,21 @@
         <v>0</v>
       </c>
       <c r="M22" s="29"/>
-      <c r="N22" s="53"/>
+      <c r="N22" s="52"/>
       <c r="O22" s="49">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P22" s="52"/>
-      <c r="Q22" s="52"/>
+      <c r="P22" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q22" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R22" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -2271,10 +2236,16 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P23" s="52"/>
-      <c r="Q23" s="52"/>
+      <c r="P23" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q23" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R23" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -2288,7 +2259,7 @@
         <v>0</v>
       </c>
       <c r="G24" s="29"/>
-      <c r="H24" s="53"/>
+      <c r="H24" s="52"/>
       <c r="I24" s="49">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -2300,15 +2271,21 @@
         <v>0</v>
       </c>
       <c r="M24" s="29"/>
-      <c r="N24" s="53"/>
+      <c r="N24" s="52"/>
       <c r="O24" s="49">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P24" s="52"/>
-      <c r="Q24" s="52"/>
+      <c r="P24" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q24" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R24" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -2339,10 +2316,16 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P25" s="52"/>
-      <c r="Q25" s="52"/>
+      <c r="P25" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q25" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R25" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -2356,7 +2339,7 @@
         <v>0</v>
       </c>
       <c r="G26" s="29"/>
-      <c r="H26" s="53"/>
+      <c r="H26" s="52"/>
       <c r="I26" s="49">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -2368,15 +2351,21 @@
         <v>0</v>
       </c>
       <c r="M26" s="29"/>
-      <c r="N26" s="53"/>
+      <c r="N26" s="52"/>
       <c r="O26" s="49">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P26" s="52"/>
-      <c r="Q26" s="52"/>
+      <c r="P26" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q26" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R26" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -2407,10 +2396,16 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P27" s="52"/>
-      <c r="Q27" s="52"/>
+      <c r="P27" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q27" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R27" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -2424,7 +2419,7 @@
         <v>0</v>
       </c>
       <c r="G28" s="29"/>
-      <c r="H28" s="53"/>
+      <c r="H28" s="52"/>
       <c r="I28" s="49">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -2436,15 +2431,21 @@
         <v>0</v>
       </c>
       <c r="M28" s="29"/>
-      <c r="N28" s="53"/>
+      <c r="N28" s="52"/>
       <c r="O28" s="49">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P28" s="52"/>
-      <c r="Q28" s="52"/>
+      <c r="P28" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q28" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R28" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -2458,7 +2459,7 @@
         <v>0</v>
       </c>
       <c r="G29" s="34"/>
-      <c r="H29" s="54"/>
+      <c r="H29" s="53"/>
       <c r="I29" s="49">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -2470,15 +2471,21 @@
         <v>0</v>
       </c>
       <c r="M29" s="34"/>
-      <c r="N29" s="54"/>
+      <c r="N29" s="53"/>
       <c r="O29" s="49">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P29" s="55"/>
-      <c r="Q29" s="55"/>
+      <c r="P29" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q29" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R29" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -2509,10 +2516,16 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P30" s="52"/>
-      <c r="Q30" s="52"/>
+      <c r="P30" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q30" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R30" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -2526,7 +2539,7 @@
         <v>0</v>
       </c>
       <c r="G31" s="29"/>
-      <c r="H31" s="53"/>
+      <c r="H31" s="52"/>
       <c r="I31" s="49">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -2538,15 +2551,21 @@
         <v>0</v>
       </c>
       <c r="M31" s="29"/>
-      <c r="N31" s="53"/>
+      <c r="N31" s="52"/>
       <c r="O31" s="49">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P31" s="52"/>
-      <c r="Q31" s="52"/>
+      <c r="P31" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q31" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R31" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -2577,10 +2596,16 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P32" s="52"/>
-      <c r="Q32" s="52"/>
+      <c r="P32" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q32" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R32" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -2611,10 +2636,16 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P33" s="52"/>
-      <c r="Q33" s="52"/>
+      <c r="P33" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q33" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R33" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -2628,7 +2659,7 @@
         <v>0</v>
       </c>
       <c r="G34" s="29"/>
-      <c r="H34" s="53"/>
+      <c r="H34" s="52"/>
       <c r="I34" s="49">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -2640,15 +2671,21 @@
         <v>0</v>
       </c>
       <c r="M34" s="29"/>
-      <c r="N34" s="53"/>
+      <c r="N34" s="52"/>
       <c r="O34" s="49">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P34" s="52"/>
-      <c r="Q34" s="52"/>
+      <c r="P34" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q34" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R34" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -2662,7 +2699,7 @@
         <v>0</v>
       </c>
       <c r="G35" s="29"/>
-      <c r="H35" s="53"/>
+      <c r="H35" s="52"/>
       <c r="I35" s="49">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -2674,15 +2711,21 @@
         <v>0</v>
       </c>
       <c r="M35" s="29"/>
-      <c r="N35" s="53"/>
+      <c r="N35" s="52"/>
       <c r="O35" s="49">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P35" s="52"/>
-      <c r="Q35" s="52"/>
+      <c r="P35" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q35" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R35" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -2713,10 +2756,16 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P36" s="52"/>
-      <c r="Q36" s="52"/>
+      <c r="P36" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q36" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R36" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -2747,10 +2796,16 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P37" s="52"/>
-      <c r="Q37" s="52"/>
+      <c r="P37" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q37" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R37" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -2781,10 +2836,16 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P38" s="56"/>
-      <c r="Q38" s="56"/>
+      <c r="P38" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q38" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R38" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -2815,10 +2876,16 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P39" s="56"/>
-      <c r="Q39" s="56"/>
+      <c r="P39" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q39" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R39" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -2849,10 +2916,16 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P40" s="52"/>
-      <c r="Q40" s="52"/>
+      <c r="P40" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q40" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R40" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -2883,10 +2956,16 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P41" s="52"/>
-      <c r="Q41" s="52"/>
+      <c r="P41" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q41" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R41" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -2917,10 +2996,16 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P42" s="56"/>
-      <c r="Q42" s="56"/>
+      <c r="P42" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q42" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R42" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -2951,10 +3036,16 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P43" s="56"/>
-      <c r="Q43" s="56"/>
+      <c r="P43" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q43" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R43" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -2968,7 +3059,7 @@
         <v>0</v>
       </c>
       <c r="G44" s="34"/>
-      <c r="H44" s="54"/>
+      <c r="H44" s="53"/>
       <c r="I44" s="49">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -2980,15 +3071,21 @@
         <v>0</v>
       </c>
       <c r="M44" s="34"/>
-      <c r="N44" s="54"/>
+      <c r="N44" s="53"/>
       <c r="O44" s="49">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P44" s="57"/>
-      <c r="Q44" s="57"/>
+      <c r="P44" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q44" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R44" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -3019,10 +3116,16 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P45" s="52"/>
-      <c r="Q45" s="52"/>
+      <c r="P45" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q45" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R45" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -3032,7 +3135,7 @@
       <c r="D46" s="23"/>
       <c r="E46" s="24"/>
       <c r="F46" s="18">
-        <f t="shared" ref="F46:F56" si="5">D46+E46</f>
+        <f t="shared" ref="F46:F56" si="7">D46+E46</f>
         <v>0</v>
       </c>
       <c r="G46" s="25"/>
@@ -3044,19 +3147,25 @@
       <c r="J46" s="25"/>
       <c r="K46" s="26"/>
       <c r="L46" s="47">
-        <f t="shared" ref="L46:L56" si="6">J46+K46</f>
+        <f t="shared" ref="L46:L56" si="8">J46+K46</f>
         <v>0</v>
       </c>
       <c r="M46" s="25"/>
       <c r="N46" s="51"/>
       <c r="O46" s="49">
-        <f t="shared" ref="O46:O56" si="7">M46+N46</f>
-        <v>0</v>
-      </c>
-      <c r="P46" s="52"/>
-      <c r="Q46" s="52"/>
+        <f t="shared" ref="O46:O56" si="9">M46+N46</f>
+        <v>0</v>
+      </c>
+      <c r="P46" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q46" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R46" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -3066,7 +3175,7 @@
       <c r="D47" s="23"/>
       <c r="E47" s="24"/>
       <c r="F47" s="18">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="G47" s="25"/>
@@ -3078,19 +3187,25 @@
       <c r="J47" s="25"/>
       <c r="K47" s="26"/>
       <c r="L47" s="47">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="M47" s="25"/>
       <c r="N47" s="51"/>
       <c r="O47" s="49">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="P47" s="52"/>
-      <c r="Q47" s="52"/>
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="P47" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q47" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R47" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -3100,7 +3215,7 @@
       <c r="D48" s="23"/>
       <c r="E48" s="24"/>
       <c r="F48" s="18">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="G48" s="25"/>
@@ -3112,19 +3227,25 @@
       <c r="J48" s="25"/>
       <c r="K48" s="26"/>
       <c r="L48" s="47">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="M48" s="25"/>
       <c r="N48" s="51"/>
       <c r="O48" s="49">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="P48" s="52"/>
-      <c r="Q48" s="52"/>
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="P48" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q48" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R48" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -3134,7 +3255,7 @@
       <c r="D49" s="37"/>
       <c r="E49" s="38"/>
       <c r="F49" s="18">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="G49" s="37"/>
@@ -3146,19 +3267,25 @@
       <c r="J49" s="37"/>
       <c r="K49" s="38"/>
       <c r="L49" s="47">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="M49" s="37"/>
       <c r="N49" s="38"/>
       <c r="O49" s="49">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="P49" s="56"/>
-      <c r="Q49" s="56"/>
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="P49" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q49" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R49" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -3168,7 +3295,7 @@
       <c r="D50" s="23"/>
       <c r="E50" s="24"/>
       <c r="F50" s="18">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="G50" s="25"/>
@@ -3180,19 +3307,25 @@
       <c r="J50" s="25"/>
       <c r="K50" s="26"/>
       <c r="L50" s="47">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="M50" s="25"/>
       <c r="N50" s="51"/>
       <c r="O50" s="49">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="P50" s="52"/>
-      <c r="Q50" s="52"/>
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="P50" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q50" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R50" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -3202,7 +3335,7 @@
       <c r="D51" s="37"/>
       <c r="E51" s="38"/>
       <c r="F51" s="18">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="G51" s="37"/>
@@ -3214,19 +3347,25 @@
       <c r="J51" s="37"/>
       <c r="K51" s="38"/>
       <c r="L51" s="47">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="M51" s="37"/>
       <c r="N51" s="38"/>
       <c r="O51" s="49">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="P51" s="56"/>
-      <c r="Q51" s="56"/>
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="P51" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q51" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R51" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -3236,7 +3375,7 @@
       <c r="D52" s="37"/>
       <c r="E52" s="38"/>
       <c r="F52" s="18">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="G52" s="37"/>
@@ -3248,19 +3387,25 @@
       <c r="J52" s="37"/>
       <c r="K52" s="38"/>
       <c r="L52" s="47">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="M52" s="37"/>
       <c r="N52" s="38"/>
       <c r="O52" s="49">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="P52" s="56"/>
-      <c r="Q52" s="56"/>
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="P52" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q52" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R52" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -3270,7 +3415,7 @@
       <c r="D53" s="23"/>
       <c r="E53" s="24"/>
       <c r="F53" s="18">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="G53" s="25"/>
@@ -3282,19 +3427,25 @@
       <c r="J53" s="25"/>
       <c r="K53" s="26"/>
       <c r="L53" s="47">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="M53" s="25"/>
       <c r="N53" s="51"/>
       <c r="O53" s="49">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="P53" s="52"/>
-      <c r="Q53" s="52"/>
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="P53" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q53" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R53" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -3304,7 +3455,7 @@
       <c r="D54" s="23"/>
       <c r="E54" s="24"/>
       <c r="F54" s="18">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="G54" s="25"/>
@@ -3316,19 +3467,25 @@
       <c r="J54" s="25"/>
       <c r="K54" s="26"/>
       <c r="L54" s="47">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="M54" s="25"/>
       <c r="N54" s="51"/>
       <c r="O54" s="49">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="P54" s="52"/>
-      <c r="Q54" s="52"/>
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="P54" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q54" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R54" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -3338,7 +3495,7 @@
       <c r="D55" s="23"/>
       <c r="E55" s="24"/>
       <c r="F55" s="18">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="G55" s="25"/>
@@ -3350,19 +3507,25 @@
       <c r="J55" s="25"/>
       <c r="K55" s="26"/>
       <c r="L55" s="47">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="M55" s="25"/>
       <c r="N55" s="51"/>
       <c r="O55" s="49">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="P55" s="52"/>
-      <c r="Q55" s="52"/>
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="P55" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q55" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R55" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -3372,7 +3535,7 @@
       <c r="D56" s="37"/>
       <c r="E56" s="38"/>
       <c r="F56" s="18">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="G56" s="37"/>
@@ -3384,27 +3547,33 @@
       <c r="J56" s="37"/>
       <c r="K56" s="38"/>
       <c r="L56" s="47">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="M56" s="37"/>
       <c r="N56" s="38"/>
       <c r="O56" s="49">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="P56" s="56"/>
-      <c r="Q56" s="56"/>
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="P56" s="50">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q56" s="50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
       <c r="R56" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
     <row r="57" spans="2:18" ht="33.75" customHeight="1" thickBot="1">
-      <c r="B57" s="74" t="s">
+      <c r="B57" s="88" t="s">
         <v>20</v>
       </c>
-      <c r="C57" s="75"/>
+      <c r="C57" s="89"/>
       <c r="D57" s="41">
         <f>SUM(D16:D56)</f>
         <v>0</v>
@@ -3414,51 +3583,55 @@
         <v>0</v>
       </c>
       <c r="F57" s="42">
-        <f t="shared" ref="F57:R57" si="8">SUM(F16:F56)</f>
+        <f t="shared" ref="F57:Q57" si="10">SUM(F16:F56)</f>
         <v>0</v>
       </c>
       <c r="G57" s="41">
+        <f>SUM(G16:G56)</f>
         <v>0</v>
       </c>
       <c r="H57" s="41">
-        <v>0</v>
-      </c>
-      <c r="I57" s="41">
-        <f>SUM(I16:I56)</f>
+        <f>SUM(H16:H56)</f>
+        <v>0</v>
+      </c>
+      <c r="I57" s="42">
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="J57" s="41">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="K57" s="41">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="L57" s="41">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="M57" s="41">
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="N57" s="41">
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="O57" s="41">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="P57" s="58">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="P57" s="54">
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="Q57" s="42">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="R57" s="50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -3490,55 +3663,55 @@
       <c r="F59" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="N59" s="67" t="s">
+      <c r="N59" s="85" t="s">
         <v>24</v>
       </c>
-      <c r="O59" s="67"/>
+      <c r="O59" s="85"/>
     </row>
     <row r="60" spans="2:18" ht="21" customHeight="1"/>
     <row r="61" spans="2:18" ht="21" customHeight="1">
       <c r="B61" s="43" t="s">
         <v>32</v>
       </c>
-      <c r="G61" s="68" t="s">
+      <c r="G61" s="86" t="s">
         <v>33</v>
       </c>
-      <c r="H61" s="68"/>
-      <c r="I61" s="68"/>
-      <c r="J61" s="68"/>
-      <c r="N61" s="69" t="s">
+      <c r="H61" s="86"/>
+      <c r="I61" s="86"/>
+      <c r="J61" s="86"/>
+      <c r="N61" s="87" t="s">
         <v>25</v>
       </c>
-      <c r="O61" s="69"/>
-      <c r="P61" s="69"/>
-      <c r="Q61" s="69"/>
+      <c r="O61" s="87"/>
+      <c r="P61" s="87"/>
+      <c r="Q61" s="87"/>
     </row>
     <row r="62" spans="2:18" ht="21" customHeight="1">
       <c r="B62" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="G62" s="79" t="s">
+      <c r="G62" s="62" t="s">
         <v>31</v>
       </c>
-      <c r="H62" s="79"/>
-      <c r="I62" s="79"/>
-      <c r="J62" s="79"/>
-      <c r="N62" s="79" t="s">
+      <c r="H62" s="62"/>
+      <c r="I62" s="62"/>
+      <c r="J62" s="62"/>
+      <c r="N62" s="62" t="s">
         <v>35</v>
       </c>
-      <c r="O62" s="79"/>
-      <c r="P62" s="79"/>
-      <c r="Q62" s="79"/>
+      <c r="O62" s="62"/>
+      <c r="P62" s="62"/>
+      <c r="Q62" s="62"/>
     </row>
     <row r="63" spans="2:18" ht="21" customHeight="1">
-      <c r="G63" s="61"/>
-      <c r="H63" s="61"/>
-      <c r="I63" s="61"/>
-      <c r="J63" s="61"/>
-      <c r="N63" s="79"/>
-      <c r="O63" s="79"/>
-      <c r="P63" s="79"/>
-      <c r="Q63" s="79"/>
+      <c r="G63" s="57"/>
+      <c r="H63" s="57"/>
+      <c r="I63" s="57"/>
+      <c r="J63" s="57"/>
+      <c r="N63" s="62"/>
+      <c r="O63" s="62"/>
+      <c r="P63" s="62"/>
+      <c r="Q63" s="62"/>
     </row>
     <row r="64" spans="2:18" ht="21" customHeight="1">
       <c r="B64" s="1" t="s">
@@ -3546,7 +3719,7 @@
       </c>
     </row>
     <row r="65" spans="2:2" ht="21" customHeight="1">
-      <c r="B65" s="59"/>
+      <c r="B65" s="55"/>
     </row>
     <row r="66" spans="2:2" ht="21" customHeight="1"/>
     <row r="67" spans="2:2" ht="21" customHeight="1"/>
@@ -3579,11 +3752,6 @@
     <mergeCell ref="P12:R14"/>
     <mergeCell ref="D13:L13"/>
     <mergeCell ref="D14:F14"/>
-    <mergeCell ref="B1:R1"/>
-    <mergeCell ref="B2:R2"/>
-    <mergeCell ref="B3:R3"/>
-    <mergeCell ref="B4:R4"/>
-    <mergeCell ref="B5:R5"/>
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="J14:L14"/>
     <mergeCell ref="G14:I14"/>
@@ -3592,6 +3760,11 @@
     <mergeCell ref="N61:Q61"/>
     <mergeCell ref="B57:C57"/>
     <mergeCell ref="D12:O12"/>
+    <mergeCell ref="B1:R1"/>
+    <mergeCell ref="B2:R2"/>
+    <mergeCell ref="B3:R3"/>
+    <mergeCell ref="B4:R4"/>
+    <mergeCell ref="B5:R5"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B4" r:id="rId1" xr:uid="{5EAE8D1D-5A31-4631-AC47-0FB40220C481}"/>

</xml_diff>

<commit_message>
var report template updated
</commit_message>
<xml_diff>
--- a/sample/VAR-REPORT.xlsx
+++ b/sample/VAR-REPORT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Miks\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04A4C52E-30AA-4CBF-A3E0-5E38AB1289A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{697047C2-A8AE-46A9-8BD1-B577A3F0046D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{39334F03-1232-460D-B301-DE63E4B3EB5C}"/>
   </bookViews>
@@ -118,9 +118,6 @@
     <t>Noted by:</t>
   </si>
   <si>
-    <t>MARIA DONNALYN E. BRIÑAS</t>
-  </si>
-  <si>
     <t>QFM-OCT-006 Rev 0 2022.02.16</t>
   </si>
   <si>
@@ -139,23 +136,26 @@
     <t>LOCAL REGISTRY COLLECTION OFFICER I</t>
   </si>
   <si>
-    <t>MIZPAH A. LENESES</t>
-  </si>
-  <si>
-    <t>ROLDAN B. AQUINO</t>
-  </si>
-  <si>
     <t>VAR 2</t>
   </si>
   <si>
     <t>City Tourism Officer                                                                   CGDH-1</t>
+  </si>
+  <si>
+    <t>______________________</t>
+  </si>
+  <si>
+    <t>____________________________</t>
+  </si>
+  <si>
+    <t>___________________________</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <name val="ＭＳ Ｐゴシック"/>
@@ -234,6 +234,11 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -832,7 +837,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0"/>
@@ -989,10 +994,6 @@
     <xf numFmtId="3" fontId="1" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -1041,7 +1042,127 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1056,128 +1177,16 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -1575,107 +1584,107 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:18" ht="15">
-      <c r="B1" s="58" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="58"/>
-      <c r="D1" s="58"/>
-      <c r="E1" s="58"/>
-      <c r="F1" s="58"/>
-      <c r="G1" s="58"/>
-      <c r="H1" s="58"/>
-      <c r="I1" s="58"/>
-      <c r="J1" s="58"/>
-      <c r="K1" s="58"/>
-      <c r="L1" s="58"/>
-      <c r="M1" s="58"/>
-      <c r="N1" s="58"/>
-      <c r="O1" s="58"/>
-      <c r="P1" s="58"/>
-      <c r="Q1" s="58"/>
-      <c r="R1" s="58"/>
+      <c r="B1" s="87" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="87"/>
+      <c r="D1" s="87"/>
+      <c r="E1" s="87"/>
+      <c r="F1" s="87"/>
+      <c r="G1" s="87"/>
+      <c r="H1" s="87"/>
+      <c r="I1" s="87"/>
+      <c r="J1" s="87"/>
+      <c r="K1" s="87"/>
+      <c r="L1" s="87"/>
+      <c r="M1" s="87"/>
+      <c r="N1" s="87"/>
+      <c r="O1" s="87"/>
+      <c r="P1" s="87"/>
+      <c r="Q1" s="87"/>
+      <c r="R1" s="87"/>
     </row>
     <row r="2" spans="2:18" ht="15">
-      <c r="B2" s="58" t="s">
+      <c r="B2" s="87" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="58"/>
-      <c r="I2" s="58"/>
-      <c r="J2" s="58"/>
-      <c r="K2" s="58"/>
-      <c r="L2" s="58"/>
-      <c r="M2" s="58"/>
-      <c r="N2" s="58"/>
-      <c r="O2" s="58"/>
-      <c r="P2" s="58"/>
-      <c r="Q2" s="58"/>
-      <c r="R2" s="58"/>
+      <c r="C2" s="87"/>
+      <c r="D2" s="87"/>
+      <c r="E2" s="87"/>
+      <c r="F2" s="87"/>
+      <c r="G2" s="87"/>
+      <c r="H2" s="87"/>
+      <c r="I2" s="87"/>
+      <c r="J2" s="87"/>
+      <c r="K2" s="87"/>
+      <c r="L2" s="87"/>
+      <c r="M2" s="87"/>
+      <c r="N2" s="87"/>
+      <c r="O2" s="87"/>
+      <c r="P2" s="87"/>
+      <c r="Q2" s="87"/>
+      <c r="R2" s="87"/>
     </row>
     <row r="3" spans="2:18">
-      <c r="B3" s="59" t="s">
+      <c r="B3" s="88" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="59"/>
-      <c r="L3" s="59"/>
-      <c r="M3" s="59"/>
-      <c r="N3" s="59"/>
-      <c r="O3" s="59"/>
-      <c r="P3" s="59"/>
-      <c r="Q3" s="59"/>
-      <c r="R3" s="59"/>
+      <c r="C3" s="88"/>
+      <c r="D3" s="88"/>
+      <c r="E3" s="88"/>
+      <c r="F3" s="88"/>
+      <c r="G3" s="88"/>
+      <c r="H3" s="88"/>
+      <c r="I3" s="88"/>
+      <c r="J3" s="88"/>
+      <c r="K3" s="88"/>
+      <c r="L3" s="88"/>
+      <c r="M3" s="88"/>
+      <c r="N3" s="88"/>
+      <c r="O3" s="88"/>
+      <c r="P3" s="88"/>
+      <c r="Q3" s="88"/>
+      <c r="R3" s="88"/>
     </row>
     <row r="4" spans="2:18">
-      <c r="B4" s="60" t="s">
+      <c r="B4" s="89" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="60"/>
-      <c r="D4" s="60"/>
-      <c r="E4" s="60"/>
-      <c r="F4" s="60"/>
-      <c r="G4" s="60"/>
-      <c r="H4" s="60"/>
-      <c r="I4" s="60"/>
-      <c r="J4" s="60"/>
-      <c r="K4" s="60"/>
-      <c r="L4" s="60"/>
-      <c r="M4" s="60"/>
-      <c r="N4" s="60"/>
-      <c r="O4" s="60"/>
-      <c r="P4" s="60"/>
-      <c r="Q4" s="60"/>
-      <c r="R4" s="60"/>
+      <c r="C4" s="89"/>
+      <c r="D4" s="89"/>
+      <c r="E4" s="89"/>
+      <c r="F4" s="89"/>
+      <c r="G4" s="89"/>
+      <c r="H4" s="89"/>
+      <c r="I4" s="89"/>
+      <c r="J4" s="89"/>
+      <c r="K4" s="89"/>
+      <c r="L4" s="89"/>
+      <c r="M4" s="89"/>
+      <c r="N4" s="89"/>
+      <c r="O4" s="89"/>
+      <c r="P4" s="89"/>
+      <c r="Q4" s="89"/>
+      <c r="R4" s="89"/>
     </row>
     <row r="5" spans="2:18" ht="15">
-      <c r="B5" s="61"/>
-      <c r="C5" s="61"/>
-      <c r="D5" s="61"/>
-      <c r="E5" s="61"/>
-      <c r="F5" s="61"/>
-      <c r="G5" s="61"/>
-      <c r="H5" s="61"/>
-      <c r="I5" s="61"/>
-      <c r="J5" s="61"/>
-      <c r="K5" s="61"/>
-      <c r="L5" s="61"/>
-      <c r="M5" s="61"/>
-      <c r="N5" s="61"/>
-      <c r="O5" s="61"/>
-      <c r="P5" s="61"/>
-      <c r="Q5" s="61"/>
-      <c r="R5" s="61"/>
+      <c r="B5" s="90"/>
+      <c r="C5" s="90"/>
+      <c r="D5" s="90"/>
+      <c r="E5" s="90"/>
+      <c r="F5" s="90"/>
+      <c r="G5" s="90"/>
+      <c r="H5" s="90"/>
+      <c r="I5" s="90"/>
+      <c r="J5" s="90"/>
+      <c r="K5" s="90"/>
+      <c r="L5" s="90"/>
+      <c r="M5" s="90"/>
+      <c r="N5" s="90"/>
+      <c r="O5" s="90"/>
+      <c r="P5" s="90"/>
+      <c r="Q5" s="90"/>
+      <c r="R5" s="90"/>
     </row>
     <row r="6" spans="2:18" ht="15">
       <c r="B6" s="2" t="s">
@@ -1697,7 +1706,7 @@
       <c r="P6" s="3"/>
       <c r="Q6" s="3"/>
       <c r="R6" s="3" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="2:18" ht="14.25" customHeight="1">
@@ -1759,7 +1768,7 @@
       <c r="O9" s="7"/>
       <c r="P9" s="7"/>
       <c r="Q9" s="7"/>
-      <c r="R9" s="45"/>
+      <c r="R9" s="44"/>
     </row>
     <row r="10" spans="2:18" ht="15.75" customHeight="1" thickBot="1">
       <c r="B10" s="3"/>
@@ -1782,7 +1791,7 @@
       <c r="O10" s="8"/>
       <c r="P10" s="8"/>
       <c r="Q10" s="8"/>
-      <c r="R10" s="45"/>
+      <c r="R10" s="44"/>
     </row>
     <row r="11" spans="2:18" ht="8.25" customHeight="1" thickBot="1">
       <c r="B11" s="3"/>
@@ -1796,93 +1805,93 @@
       <c r="J11" s="9"/>
       <c r="K11" s="9"/>
       <c r="L11" s="9"/>
-      <c r="M11" s="45"/>
-      <c r="N11" s="45"/>
-      <c r="O11" s="45"/>
+      <c r="M11" s="44"/>
+      <c r="N11" s="44"/>
+      <c r="O11" s="44"/>
       <c r="P11" s="9"/>
       <c r="Q11" s="9"/>
       <c r="R11" s="9"/>
     </row>
     <row r="12" spans="2:18" ht="16.5" customHeight="1">
-      <c r="B12" s="83" t="s">
+      <c r="B12" s="77" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="84"/>
-      <c r="D12" s="90" t="s">
+      <c r="C12" s="78"/>
+      <c r="D12" s="84" t="s">
         <v>10</v>
       </c>
-      <c r="E12" s="91"/>
-      <c r="F12" s="91"/>
-      <c r="G12" s="91"/>
-      <c r="H12" s="91"/>
-      <c r="I12" s="91"/>
-      <c r="J12" s="91"/>
-      <c r="K12" s="91"/>
-      <c r="L12" s="91"/>
-      <c r="M12" s="91"/>
-      <c r="N12" s="91"/>
-      <c r="O12" s="92"/>
-      <c r="P12" s="71" t="s">
+      <c r="E12" s="85"/>
+      <c r="F12" s="85"/>
+      <c r="G12" s="85"/>
+      <c r="H12" s="85"/>
+      <c r="I12" s="85"/>
+      <c r="J12" s="85"/>
+      <c r="K12" s="85"/>
+      <c r="L12" s="85"/>
+      <c r="M12" s="85"/>
+      <c r="N12" s="85"/>
+      <c r="O12" s="86"/>
+      <c r="P12" s="67" t="s">
         <v>11</v>
       </c>
-      <c r="Q12" s="72"/>
-      <c r="R12" s="73"/>
+      <c r="Q12" s="68"/>
+      <c r="R12" s="69"/>
     </row>
     <row r="13" spans="2:18" ht="15" customHeight="1">
-      <c r="B13" s="63" t="s">
+      <c r="B13" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="66" t="s">
+      <c r="C13" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="D13" s="78" t="s">
+      <c r="D13" s="72" t="s">
         <v>14</v>
       </c>
-      <c r="E13" s="79"/>
-      <c r="F13" s="79"/>
-      <c r="G13" s="79"/>
-      <c r="H13" s="79"/>
-      <c r="I13" s="79"/>
-      <c r="J13" s="79"/>
-      <c r="K13" s="79"/>
-      <c r="L13" s="79"/>
-      <c r="M13" s="63" t="s">
+      <c r="E13" s="73"/>
+      <c r="F13" s="73"/>
+      <c r="G13" s="73"/>
+      <c r="H13" s="73"/>
+      <c r="I13" s="73"/>
+      <c r="J13" s="73"/>
+      <c r="K13" s="73"/>
+      <c r="L13" s="73"/>
+      <c r="M13" s="57" t="s">
         <v>15</v>
       </c>
-      <c r="N13" s="69"/>
-      <c r="O13" s="70"/>
-      <c r="P13" s="64"/>
-      <c r="Q13" s="74"/>
-      <c r="R13" s="75"/>
+      <c r="N13" s="63"/>
+      <c r="O13" s="64"/>
+      <c r="P13" s="58"/>
+      <c r="Q13" s="70"/>
+      <c r="R13" s="71"/>
     </row>
     <row r="14" spans="2:18" ht="28.5" customHeight="1" thickBot="1">
-      <c r="B14" s="64"/>
-      <c r="C14" s="67"/>
-      <c r="D14" s="80" t="s">
+      <c r="B14" s="58"/>
+      <c r="C14" s="61"/>
+      <c r="D14" s="74" t="s">
+        <v>26</v>
+      </c>
+      <c r="E14" s="75"/>
+      <c r="F14" s="76"/>
+      <c r="G14" s="74" t="s">
         <v>27</v>
       </c>
-      <c r="E14" s="81"/>
-      <c r="F14" s="82"/>
-      <c r="G14" s="80" t="s">
+      <c r="H14" s="75"/>
+      <c r="I14" s="76"/>
+      <c r="J14" s="74" t="s">
         <v>28</v>
       </c>
-      <c r="H14" s="81"/>
-      <c r="I14" s="82"/>
-      <c r="J14" s="80" t="s">
-        <v>29</v>
-      </c>
-      <c r="K14" s="81"/>
-      <c r="L14" s="82"/>
-      <c r="M14" s="65"/>
-      <c r="N14" s="76"/>
-      <c r="O14" s="77"/>
-      <c r="P14" s="65"/>
-      <c r="Q14" s="76"/>
-      <c r="R14" s="77"/>
+      <c r="K14" s="75"/>
+      <c r="L14" s="76"/>
+      <c r="M14" s="59"/>
+      <c r="N14" s="65"/>
+      <c r="O14" s="66"/>
+      <c r="P14" s="59"/>
+      <c r="Q14" s="65"/>
+      <c r="R14" s="66"/>
     </row>
     <row r="15" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
-      <c r="B15" s="65"/>
-      <c r="C15" s="68"/>
+      <c r="B15" s="59"/>
+      <c r="C15" s="62"/>
       <c r="D15" s="10" t="s">
         <v>16</v>
       </c>
@@ -1892,13 +1901,13 @@
       <c r="F15" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="G15" s="56" t="s">
+      <c r="G15" s="55" t="s">
         <v>16</v>
       </c>
-      <c r="H15" s="56" t="s">
+      <c r="H15" s="55" t="s">
         <v>17</v>
       </c>
-      <c r="I15" s="56" t="s">
+      <c r="I15" s="55" t="s">
         <v>18</v>
       </c>
       <c r="J15" s="10" t="s">
@@ -1916,7 +1925,7 @@
       <c r="N15" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="O15" s="46" t="s">
+      <c r="O15" s="45" t="s">
         <v>18</v>
       </c>
       <c r="P15" s="12" t="s">
@@ -1939,32 +1948,32 @@
         <v>0</v>
       </c>
       <c r="G16" s="19"/>
-      <c r="H16" s="48"/>
-      <c r="I16" s="49">
+      <c r="H16" s="47"/>
+      <c r="I16" s="48">
         <f t="shared" ref="I16:I56" si="1">G16+H16</f>
         <v>0</v>
       </c>
       <c r="J16" s="19"/>
       <c r="K16" s="20"/>
-      <c r="L16" s="47">
+      <c r="L16" s="46">
         <f t="shared" ref="L16:L45" si="2">J16+K16</f>
         <v>0</v>
       </c>
       <c r="M16" s="19"/>
-      <c r="N16" s="48"/>
-      <c r="O16" s="49">
+      <c r="N16" s="47"/>
+      <c r="O16" s="48">
         <f t="shared" ref="O16:O45" si="3">M16+N16</f>
         <v>0</v>
       </c>
-      <c r="P16" s="50">
+      <c r="P16" s="49">
         <f>D16+G16+J16+M16</f>
         <v>0</v>
       </c>
-      <c r="Q16" s="50">
+      <c r="Q16" s="49">
         <f>E16+H16+K16+N16</f>
         <v>0</v>
       </c>
-      <c r="R16" s="50">
+      <c r="R16" s="49">
         <f>F16+I16+L16+O16</f>
         <v>0</v>
       </c>
@@ -1979,32 +1988,32 @@
         <v>0</v>
       </c>
       <c r="G17" s="25"/>
-      <c r="H17" s="51"/>
-      <c r="I17" s="49">
+      <c r="H17" s="50"/>
+      <c r="I17" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J17" s="25"/>
       <c r="K17" s="26"/>
-      <c r="L17" s="47">
+      <c r="L17" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M17" s="25"/>
-      <c r="N17" s="51"/>
-      <c r="O17" s="49">
+      <c r="N17" s="50"/>
+      <c r="O17" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P17" s="50">
+      <c r="P17" s="49">
         <f t="shared" ref="P17:P56" si="4">D17+G17+J17+M17</f>
         <v>0</v>
       </c>
-      <c r="Q17" s="50">
+      <c r="Q17" s="49">
         <f t="shared" ref="Q17:Q56" si="5">E17+H17+K17+N17</f>
         <v>0</v>
       </c>
-      <c r="R17" s="50">
+      <c r="R17" s="49">
         <f t="shared" ref="R17:R57" si="6">F17+I17+L17+O17</f>
         <v>0</v>
       </c>
@@ -2019,32 +2028,32 @@
         <v>0</v>
       </c>
       <c r="G18" s="25"/>
-      <c r="H18" s="51"/>
-      <c r="I18" s="49">
+      <c r="H18" s="50"/>
+      <c r="I18" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J18" s="25"/>
       <c r="K18" s="26"/>
-      <c r="L18" s="47">
+      <c r="L18" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M18" s="25"/>
-      <c r="N18" s="51"/>
-      <c r="O18" s="49">
+      <c r="N18" s="50"/>
+      <c r="O18" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P18" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q18" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R18" s="50">
+      <c r="P18" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q18" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R18" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -2059,32 +2068,32 @@
         <v>0</v>
       </c>
       <c r="G19" s="29"/>
-      <c r="H19" s="52"/>
-      <c r="I19" s="49">
+      <c r="H19" s="51"/>
+      <c r="I19" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J19" s="29"/>
       <c r="K19" s="30"/>
-      <c r="L19" s="47">
+      <c r="L19" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M19" s="29"/>
-      <c r="N19" s="52"/>
-      <c r="O19" s="49">
+      <c r="N19" s="51"/>
+      <c r="O19" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P19" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q19" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R19" s="50">
+      <c r="P19" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q19" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R19" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -2099,32 +2108,32 @@
         <v>0</v>
       </c>
       <c r="G20" s="29"/>
-      <c r="H20" s="52"/>
-      <c r="I20" s="49">
+      <c r="H20" s="51"/>
+      <c r="I20" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J20" s="29"/>
       <c r="K20" s="30"/>
-      <c r="L20" s="47">
+      <c r="L20" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M20" s="29"/>
-      <c r="N20" s="52"/>
-      <c r="O20" s="49">
+      <c r="N20" s="51"/>
+      <c r="O20" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P20" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q20" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R20" s="50">
+      <c r="P20" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q20" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R20" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -2139,32 +2148,32 @@
         <v>0</v>
       </c>
       <c r="G21" s="29"/>
-      <c r="H21" s="52"/>
-      <c r="I21" s="49">
+      <c r="H21" s="51"/>
+      <c r="I21" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J21" s="29"/>
       <c r="K21" s="30"/>
-      <c r="L21" s="47">
+      <c r="L21" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M21" s="29"/>
-      <c r="N21" s="52"/>
-      <c r="O21" s="49">
+      <c r="N21" s="51"/>
+      <c r="O21" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P21" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q21" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R21" s="50">
+      <c r="P21" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q21" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R21" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -2179,32 +2188,32 @@
         <v>0</v>
       </c>
       <c r="G22" s="29"/>
-      <c r="H22" s="52"/>
-      <c r="I22" s="49">
+      <c r="H22" s="51"/>
+      <c r="I22" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J22" s="29"/>
       <c r="K22" s="30"/>
-      <c r="L22" s="47">
+      <c r="L22" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M22" s="29"/>
-      <c r="N22" s="52"/>
-      <c r="O22" s="49">
+      <c r="N22" s="51"/>
+      <c r="O22" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P22" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q22" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R22" s="50">
+      <c r="P22" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q22" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R22" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -2219,32 +2228,32 @@
         <v>0</v>
       </c>
       <c r="G23" s="25"/>
-      <c r="H23" s="51"/>
-      <c r="I23" s="49">
+      <c r="H23" s="50"/>
+      <c r="I23" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J23" s="25"/>
       <c r="K23" s="26"/>
-      <c r="L23" s="47">
+      <c r="L23" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M23" s="25"/>
-      <c r="N23" s="51"/>
-      <c r="O23" s="49">
+      <c r="N23" s="50"/>
+      <c r="O23" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P23" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q23" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R23" s="50">
+      <c r="P23" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q23" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R23" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -2259,32 +2268,32 @@
         <v>0</v>
       </c>
       <c r="G24" s="29"/>
-      <c r="H24" s="52"/>
-      <c r="I24" s="49">
+      <c r="H24" s="51"/>
+      <c r="I24" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J24" s="29"/>
       <c r="K24" s="30"/>
-      <c r="L24" s="47">
+      <c r="L24" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M24" s="29"/>
-      <c r="N24" s="52"/>
-      <c r="O24" s="49">
+      <c r="N24" s="51"/>
+      <c r="O24" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P24" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q24" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R24" s="50">
+      <c r="P24" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q24" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R24" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -2299,32 +2308,32 @@
         <v>0</v>
       </c>
       <c r="G25" s="25"/>
-      <c r="H25" s="51"/>
-      <c r="I25" s="49">
+      <c r="H25" s="50"/>
+      <c r="I25" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J25" s="25"/>
       <c r="K25" s="26"/>
-      <c r="L25" s="47">
+      <c r="L25" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M25" s="25"/>
-      <c r="N25" s="51"/>
-      <c r="O25" s="49">
+      <c r="N25" s="50"/>
+      <c r="O25" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P25" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q25" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R25" s="50">
+      <c r="P25" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q25" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R25" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -2339,32 +2348,32 @@
         <v>0</v>
       </c>
       <c r="G26" s="29"/>
-      <c r="H26" s="52"/>
-      <c r="I26" s="49">
+      <c r="H26" s="51"/>
+      <c r="I26" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J26" s="29"/>
       <c r="K26" s="30"/>
-      <c r="L26" s="47">
+      <c r="L26" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M26" s="29"/>
-      <c r="N26" s="52"/>
-      <c r="O26" s="49">
+      <c r="N26" s="51"/>
+      <c r="O26" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P26" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q26" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R26" s="50">
+      <c r="P26" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q26" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R26" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -2379,32 +2388,32 @@
         <v>0</v>
       </c>
       <c r="G27" s="25"/>
-      <c r="H27" s="51"/>
-      <c r="I27" s="49">
+      <c r="H27" s="50"/>
+      <c r="I27" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J27" s="25"/>
       <c r="K27" s="26"/>
-      <c r="L27" s="47">
+      <c r="L27" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M27" s="25"/>
-      <c r="N27" s="51"/>
-      <c r="O27" s="49">
+      <c r="N27" s="50"/>
+      <c r="O27" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P27" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q27" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R27" s="50">
+      <c r="P27" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q27" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R27" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -2419,32 +2428,32 @@
         <v>0</v>
       </c>
       <c r="G28" s="29"/>
-      <c r="H28" s="52"/>
-      <c r="I28" s="49">
+      <c r="H28" s="51"/>
+      <c r="I28" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J28" s="29"/>
       <c r="K28" s="30"/>
-      <c r="L28" s="47">
+      <c r="L28" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M28" s="29"/>
-      <c r="N28" s="52"/>
-      <c r="O28" s="49">
+      <c r="N28" s="51"/>
+      <c r="O28" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P28" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q28" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R28" s="50">
+      <c r="P28" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q28" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R28" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -2459,32 +2468,32 @@
         <v>0</v>
       </c>
       <c r="G29" s="34"/>
-      <c r="H29" s="53"/>
-      <c r="I29" s="49">
+      <c r="H29" s="52"/>
+      <c r="I29" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J29" s="34"/>
       <c r="K29" s="35"/>
-      <c r="L29" s="47">
+      <c r="L29" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M29" s="34"/>
-      <c r="N29" s="53"/>
-      <c r="O29" s="49">
+      <c r="N29" s="52"/>
+      <c r="O29" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P29" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q29" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R29" s="50">
+      <c r="P29" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q29" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R29" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -2499,32 +2508,32 @@
         <v>0</v>
       </c>
       <c r="G30" s="25"/>
-      <c r="H30" s="51"/>
-      <c r="I30" s="49">
+      <c r="H30" s="50"/>
+      <c r="I30" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J30" s="25"/>
       <c r="K30" s="26"/>
-      <c r="L30" s="47">
+      <c r="L30" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M30" s="25"/>
-      <c r="N30" s="51"/>
-      <c r="O30" s="49">
+      <c r="N30" s="50"/>
+      <c r="O30" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P30" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q30" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R30" s="50">
+      <c r="P30" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q30" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R30" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -2539,32 +2548,32 @@
         <v>0</v>
       </c>
       <c r="G31" s="29"/>
-      <c r="H31" s="52"/>
-      <c r="I31" s="49">
+      <c r="H31" s="51"/>
+      <c r="I31" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J31" s="29"/>
       <c r="K31" s="30"/>
-      <c r="L31" s="47">
+      <c r="L31" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M31" s="29"/>
-      <c r="N31" s="52"/>
-      <c r="O31" s="49">
+      <c r="N31" s="51"/>
+      <c r="O31" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P31" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q31" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R31" s="50">
+      <c r="P31" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q31" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R31" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -2579,32 +2588,32 @@
         <v>0</v>
       </c>
       <c r="G32" s="25"/>
-      <c r="H32" s="51"/>
-      <c r="I32" s="49">
+      <c r="H32" s="50"/>
+      <c r="I32" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J32" s="25"/>
       <c r="K32" s="26"/>
-      <c r="L32" s="47">
+      <c r="L32" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M32" s="25"/>
-      <c r="N32" s="51"/>
-      <c r="O32" s="49">
+      <c r="N32" s="50"/>
+      <c r="O32" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P32" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q32" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R32" s="50">
+      <c r="P32" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q32" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R32" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -2619,32 +2628,32 @@
         <v>0</v>
       </c>
       <c r="G33" s="25"/>
-      <c r="H33" s="51"/>
-      <c r="I33" s="49">
+      <c r="H33" s="50"/>
+      <c r="I33" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J33" s="25"/>
       <c r="K33" s="26"/>
-      <c r="L33" s="47">
+      <c r="L33" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M33" s="25"/>
-      <c r="N33" s="51"/>
-      <c r="O33" s="49">
+      <c r="N33" s="50"/>
+      <c r="O33" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P33" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q33" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R33" s="50">
+      <c r="P33" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q33" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R33" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -2659,32 +2668,32 @@
         <v>0</v>
       </c>
       <c r="G34" s="29"/>
-      <c r="H34" s="52"/>
-      <c r="I34" s="49">
+      <c r="H34" s="51"/>
+      <c r="I34" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J34" s="29"/>
       <c r="K34" s="30"/>
-      <c r="L34" s="47">
+      <c r="L34" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M34" s="29"/>
-      <c r="N34" s="52"/>
-      <c r="O34" s="49">
+      <c r="N34" s="51"/>
+      <c r="O34" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P34" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q34" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R34" s="50">
+      <c r="P34" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q34" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R34" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -2699,32 +2708,32 @@
         <v>0</v>
       </c>
       <c r="G35" s="29"/>
-      <c r="H35" s="52"/>
-      <c r="I35" s="49">
+      <c r="H35" s="51"/>
+      <c r="I35" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J35" s="29"/>
       <c r="K35" s="30"/>
-      <c r="L35" s="47">
+      <c r="L35" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M35" s="29"/>
-      <c r="N35" s="52"/>
-      <c r="O35" s="49">
+      <c r="N35" s="51"/>
+      <c r="O35" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P35" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q35" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R35" s="50">
+      <c r="P35" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q35" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R35" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -2739,32 +2748,32 @@
         <v>0</v>
       </c>
       <c r="G36" s="25"/>
-      <c r="H36" s="51"/>
-      <c r="I36" s="49">
+      <c r="H36" s="50"/>
+      <c r="I36" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J36" s="25"/>
       <c r="K36" s="26"/>
-      <c r="L36" s="47">
+      <c r="L36" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M36" s="25"/>
-      <c r="N36" s="51"/>
-      <c r="O36" s="49">
+      <c r="N36" s="50"/>
+      <c r="O36" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P36" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q36" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R36" s="50">
+      <c r="P36" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q36" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R36" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -2779,32 +2788,32 @@
         <v>0</v>
       </c>
       <c r="G37" s="25"/>
-      <c r="H37" s="51"/>
-      <c r="I37" s="49">
+      <c r="H37" s="50"/>
+      <c r="I37" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J37" s="25"/>
       <c r="K37" s="26"/>
-      <c r="L37" s="47">
+      <c r="L37" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M37" s="25"/>
-      <c r="N37" s="51"/>
-      <c r="O37" s="49">
+      <c r="N37" s="50"/>
+      <c r="O37" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P37" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q37" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R37" s="50">
+      <c r="P37" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q37" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R37" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -2820,31 +2829,31 @@
       </c>
       <c r="G38" s="37"/>
       <c r="H38" s="38"/>
-      <c r="I38" s="49">
+      <c r="I38" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J38" s="37"/>
       <c r="K38" s="38"/>
-      <c r="L38" s="47">
+      <c r="L38" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M38" s="37"/>
       <c r="N38" s="38"/>
-      <c r="O38" s="49">
+      <c r="O38" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P38" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q38" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R38" s="50">
+      <c r="P38" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q38" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R38" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -2860,31 +2869,31 @@
       </c>
       <c r="G39" s="37"/>
       <c r="H39" s="38"/>
-      <c r="I39" s="49">
+      <c r="I39" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J39" s="37"/>
       <c r="K39" s="38"/>
-      <c r="L39" s="47">
+      <c r="L39" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M39" s="37"/>
       <c r="N39" s="38"/>
-      <c r="O39" s="49">
+      <c r="O39" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P39" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q39" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R39" s="50">
+      <c r="P39" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q39" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R39" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -2899,32 +2908,32 @@
         <v>0</v>
       </c>
       <c r="G40" s="25"/>
-      <c r="H40" s="51"/>
-      <c r="I40" s="49">
+      <c r="H40" s="50"/>
+      <c r="I40" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J40" s="25"/>
       <c r="K40" s="26"/>
-      <c r="L40" s="47">
+      <c r="L40" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M40" s="25"/>
-      <c r="N40" s="51"/>
-      <c r="O40" s="49">
+      <c r="N40" s="50"/>
+      <c r="O40" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P40" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q40" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R40" s="50">
+      <c r="P40" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q40" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R40" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -2939,32 +2948,32 @@
         <v>0</v>
       </c>
       <c r="G41" s="25"/>
-      <c r="H41" s="51"/>
-      <c r="I41" s="49">
+      <c r="H41" s="50"/>
+      <c r="I41" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J41" s="25"/>
       <c r="K41" s="26"/>
-      <c r="L41" s="47">
+      <c r="L41" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M41" s="25"/>
-      <c r="N41" s="51"/>
-      <c r="O41" s="49">
+      <c r="N41" s="50"/>
+      <c r="O41" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P41" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q41" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R41" s="50">
+      <c r="P41" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q41" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R41" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -2980,31 +2989,31 @@
       </c>
       <c r="G42" s="37"/>
       <c r="H42" s="38"/>
-      <c r="I42" s="49">
+      <c r="I42" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J42" s="37"/>
       <c r="K42" s="38"/>
-      <c r="L42" s="47">
+      <c r="L42" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M42" s="37"/>
       <c r="N42" s="38"/>
-      <c r="O42" s="49">
+      <c r="O42" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P42" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q42" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R42" s="50">
+      <c r="P42" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q42" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R42" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -3020,31 +3029,31 @@
       </c>
       <c r="G43" s="37"/>
       <c r="H43" s="38"/>
-      <c r="I43" s="49">
+      <c r="I43" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J43" s="37"/>
       <c r="K43" s="38"/>
-      <c r="L43" s="47">
+      <c r="L43" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M43" s="37"/>
       <c r="N43" s="38"/>
-      <c r="O43" s="49">
+      <c r="O43" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P43" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q43" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R43" s="50">
+      <c r="P43" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q43" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R43" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -3059,32 +3068,32 @@
         <v>0</v>
       </c>
       <c r="G44" s="34"/>
-      <c r="H44" s="53"/>
-      <c r="I44" s="49">
+      <c r="H44" s="52"/>
+      <c r="I44" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J44" s="34"/>
       <c r="K44" s="35"/>
-      <c r="L44" s="47">
+      <c r="L44" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M44" s="34"/>
-      <c r="N44" s="53"/>
-      <c r="O44" s="49">
+      <c r="N44" s="52"/>
+      <c r="O44" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P44" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q44" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R44" s="50">
+      <c r="P44" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q44" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R44" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -3099,32 +3108,32 @@
         <v>0</v>
       </c>
       <c r="G45" s="25"/>
-      <c r="H45" s="51"/>
-      <c r="I45" s="49">
+      <c r="H45" s="50"/>
+      <c r="I45" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J45" s="25"/>
       <c r="K45" s="26"/>
-      <c r="L45" s="47">
+      <c r="L45" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M45" s="25"/>
-      <c r="N45" s="51"/>
-      <c r="O45" s="49">
+      <c r="N45" s="50"/>
+      <c r="O45" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P45" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q45" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R45" s="50">
+      <c r="P45" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q45" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R45" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -3139,32 +3148,32 @@
         <v>0</v>
       </c>
       <c r="G46" s="25"/>
-      <c r="H46" s="51"/>
-      <c r="I46" s="49">
+      <c r="H46" s="50"/>
+      <c r="I46" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J46" s="25"/>
       <c r="K46" s="26"/>
-      <c r="L46" s="47">
+      <c r="L46" s="46">
         <f t="shared" ref="L46:L56" si="8">J46+K46</f>
         <v>0</v>
       </c>
       <c r="M46" s="25"/>
-      <c r="N46" s="51"/>
-      <c r="O46" s="49">
+      <c r="N46" s="50"/>
+      <c r="O46" s="48">
         <f t="shared" ref="O46:O56" si="9">M46+N46</f>
         <v>0</v>
       </c>
-      <c r="P46" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q46" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R46" s="50">
+      <c r="P46" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q46" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R46" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -3179,32 +3188,32 @@
         <v>0</v>
       </c>
       <c r="G47" s="25"/>
-      <c r="H47" s="51"/>
-      <c r="I47" s="49">
+      <c r="H47" s="50"/>
+      <c r="I47" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J47" s="25"/>
       <c r="K47" s="26"/>
-      <c r="L47" s="47">
+      <c r="L47" s="46">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="M47" s="25"/>
-      <c r="N47" s="51"/>
-      <c r="O47" s="49">
+      <c r="N47" s="50"/>
+      <c r="O47" s="48">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="P47" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q47" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R47" s="50">
+      <c r="P47" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q47" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R47" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -3219,32 +3228,32 @@
         <v>0</v>
       </c>
       <c r="G48" s="25"/>
-      <c r="H48" s="51"/>
-      <c r="I48" s="49">
+      <c r="H48" s="50"/>
+      <c r="I48" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J48" s="25"/>
       <c r="K48" s="26"/>
-      <c r="L48" s="47">
+      <c r="L48" s="46">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="M48" s="25"/>
-      <c r="N48" s="51"/>
-      <c r="O48" s="49">
+      <c r="N48" s="50"/>
+      <c r="O48" s="48">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="P48" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q48" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R48" s="50">
+      <c r="P48" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q48" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R48" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -3260,31 +3269,31 @@
       </c>
       <c r="G49" s="37"/>
       <c r="H49" s="38"/>
-      <c r="I49" s="49">
+      <c r="I49" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J49" s="37"/>
       <c r="K49" s="38"/>
-      <c r="L49" s="47">
+      <c r="L49" s="46">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="M49" s="37"/>
       <c r="N49" s="38"/>
-      <c r="O49" s="49">
+      <c r="O49" s="48">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="P49" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q49" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R49" s="50">
+      <c r="P49" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q49" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R49" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -3299,32 +3308,32 @@
         <v>0</v>
       </c>
       <c r="G50" s="25"/>
-      <c r="H50" s="51"/>
-      <c r="I50" s="49">
+      <c r="H50" s="50"/>
+      <c r="I50" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J50" s="25"/>
       <c r="K50" s="26"/>
-      <c r="L50" s="47">
+      <c r="L50" s="46">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="M50" s="25"/>
-      <c r="N50" s="51"/>
-      <c r="O50" s="49">
+      <c r="N50" s="50"/>
+      <c r="O50" s="48">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="P50" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q50" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R50" s="50">
+      <c r="P50" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q50" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R50" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -3340,31 +3349,31 @@
       </c>
       <c r="G51" s="37"/>
       <c r="H51" s="38"/>
-      <c r="I51" s="49">
+      <c r="I51" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J51" s="37"/>
       <c r="K51" s="38"/>
-      <c r="L51" s="47">
+      <c r="L51" s="46">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="M51" s="37"/>
       <c r="N51" s="38"/>
-      <c r="O51" s="49">
+      <c r="O51" s="48">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="P51" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q51" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R51" s="50">
+      <c r="P51" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q51" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R51" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -3380,31 +3389,31 @@
       </c>
       <c r="G52" s="37"/>
       <c r="H52" s="38"/>
-      <c r="I52" s="49">
+      <c r="I52" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J52" s="37"/>
       <c r="K52" s="38"/>
-      <c r="L52" s="47">
+      <c r="L52" s="46">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="M52" s="37"/>
       <c r="N52" s="38"/>
-      <c r="O52" s="49">
+      <c r="O52" s="48">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="P52" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q52" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R52" s="50">
+      <c r="P52" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q52" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R52" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -3419,32 +3428,32 @@
         <v>0</v>
       </c>
       <c r="G53" s="25"/>
-      <c r="H53" s="51"/>
-      <c r="I53" s="49">
+      <c r="H53" s="50"/>
+      <c r="I53" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J53" s="25"/>
       <c r="K53" s="26"/>
-      <c r="L53" s="47">
+      <c r="L53" s="46">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="M53" s="25"/>
-      <c r="N53" s="51"/>
-      <c r="O53" s="49">
+      <c r="N53" s="50"/>
+      <c r="O53" s="48">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="P53" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q53" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R53" s="50">
+      <c r="P53" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q53" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R53" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -3459,32 +3468,32 @@
         <v>0</v>
       </c>
       <c r="G54" s="25"/>
-      <c r="H54" s="51"/>
-      <c r="I54" s="49">
+      <c r="H54" s="50"/>
+      <c r="I54" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J54" s="25"/>
       <c r="K54" s="26"/>
-      <c r="L54" s="47">
+      <c r="L54" s="46">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="M54" s="25"/>
-      <c r="N54" s="51"/>
-      <c r="O54" s="49">
+      <c r="N54" s="50"/>
+      <c r="O54" s="48">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="P54" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q54" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R54" s="50">
+      <c r="P54" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q54" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R54" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -3499,32 +3508,32 @@
         <v>0</v>
       </c>
       <c r="G55" s="25"/>
-      <c r="H55" s="51"/>
-      <c r="I55" s="49">
+      <c r="H55" s="50"/>
+      <c r="I55" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J55" s="25"/>
       <c r="K55" s="26"/>
-      <c r="L55" s="47">
+      <c r="L55" s="46">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="M55" s="25"/>
-      <c r="N55" s="51"/>
-      <c r="O55" s="49">
+      <c r="N55" s="50"/>
+      <c r="O55" s="48">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="P55" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q55" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R55" s="50">
+      <c r="P55" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q55" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R55" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -3540,40 +3549,40 @@
       </c>
       <c r="G56" s="37"/>
       <c r="H56" s="38"/>
-      <c r="I56" s="49">
+      <c r="I56" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J56" s="37"/>
       <c r="K56" s="38"/>
-      <c r="L56" s="47">
+      <c r="L56" s="46">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="M56" s="37"/>
       <c r="N56" s="38"/>
-      <c r="O56" s="49">
+      <c r="O56" s="48">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="P56" s="50">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q56" s="50">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R56" s="50">
+      <c r="P56" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q56" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R56" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
     <row r="57" spans="2:18" ht="33.75" customHeight="1" thickBot="1">
-      <c r="B57" s="88" t="s">
+      <c r="B57" s="82" t="s">
         <v>20</v>
       </c>
-      <c r="C57" s="89"/>
+      <c r="C57" s="83"/>
       <c r="D57" s="41">
         <f>SUM(D16:D56)</f>
         <v>0</v>
@@ -3622,7 +3631,7 @@
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="P57" s="54">
+      <c r="P57" s="53">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
@@ -3630,7 +3639,7 @@
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="R57" s="50">
+      <c r="R57" s="49">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -3663,63 +3672,63 @@
       <c r="F59" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="N59" s="85" t="s">
+      <c r="N59" s="79" t="s">
         <v>24</v>
       </c>
-      <c r="O59" s="85"/>
+      <c r="O59" s="79"/>
     </row>
     <row r="60" spans="2:18" ht="21" customHeight="1"/>
     <row r="61" spans="2:18" ht="21" customHeight="1">
-      <c r="B61" s="43" t="s">
+      <c r="B61" s="91" t="s">
+        <v>33</v>
+      </c>
+      <c r="G61" s="92" t="s">
+        <v>34</v>
+      </c>
+      <c r="H61" s="80"/>
+      <c r="I61" s="80"/>
+      <c r="J61" s="80"/>
+      <c r="N61" s="93" t="s">
+        <v>35</v>
+      </c>
+      <c r="O61" s="81"/>
+      <c r="P61" s="81"/>
+      <c r="Q61" s="81"/>
+    </row>
+    <row r="62" spans="2:18" ht="21" customHeight="1">
+      <c r="B62" s="43" t="s">
+        <v>29</v>
+      </c>
+      <c r="G62" s="56" t="s">
+        <v>30</v>
+      </c>
+      <c r="H62" s="56"/>
+      <c r="I62" s="56"/>
+      <c r="J62" s="56"/>
+      <c r="N62" s="56" t="s">
         <v>32</v>
       </c>
-      <c r="G61" s="86" t="s">
-        <v>33</v>
-      </c>
-      <c r="H61" s="86"/>
-      <c r="I61" s="86"/>
-      <c r="J61" s="86"/>
-      <c r="N61" s="87" t="s">
-        <v>25</v>
-      </c>
-      <c r="O61" s="87"/>
-      <c r="P61" s="87"/>
-      <c r="Q61" s="87"/>
-    </row>
-    <row r="62" spans="2:18" ht="21" customHeight="1">
-      <c r="B62" s="44" t="s">
-        <v>30</v>
-      </c>
-      <c r="G62" s="62" t="s">
-        <v>31</v>
-      </c>
-      <c r="H62" s="62"/>
-      <c r="I62" s="62"/>
-      <c r="J62" s="62"/>
-      <c r="N62" s="62" t="s">
-        <v>35</v>
-      </c>
-      <c r="O62" s="62"/>
-      <c r="P62" s="62"/>
-      <c r="Q62" s="62"/>
+      <c r="O62" s="56"/>
+      <c r="P62" s="56"/>
+      <c r="Q62" s="56"/>
     </row>
     <row r="63" spans="2:18" ht="21" customHeight="1">
-      <c r="G63" s="57"/>
-      <c r="H63" s="57"/>
-      <c r="I63" s="57"/>
-      <c r="J63" s="57"/>
-      <c r="N63" s="62"/>
-      <c r="O63" s="62"/>
-      <c r="P63" s="62"/>
-      <c r="Q63" s="62"/>
+      <c r="G63" s="56"/>
+      <c r="H63" s="56"/>
+      <c r="I63" s="56"/>
+      <c r="J63" s="56"/>
+      <c r="N63" s="56"/>
+      <c r="O63" s="56"/>
+      <c r="P63" s="56"/>
+      <c r="Q63" s="56"/>
     </row>
     <row r="64" spans="2:18" ht="21" customHeight="1">
       <c r="B64" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="65" spans="2:2" ht="21" customHeight="1">
-      <c r="B65" s="55"/>
+      <c r="B65" s="54"/>
     </row>
     <row r="66" spans="2:2" ht="21" customHeight="1"/>
     <row r="67" spans="2:2" ht="21" customHeight="1"/>
@@ -3744,7 +3753,12 @@
     <row r="86" ht="21" customHeight="1"/>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="G62:J62"/>
+    <mergeCell ref="G62:J63"/>
+    <mergeCell ref="B1:R1"/>
+    <mergeCell ref="B2:R2"/>
+    <mergeCell ref="B3:R3"/>
+    <mergeCell ref="B4:R4"/>
+    <mergeCell ref="B5:R5"/>
     <mergeCell ref="B13:B15"/>
     <mergeCell ref="C13:C15"/>
     <mergeCell ref="N62:Q63"/>
@@ -3760,11 +3774,6 @@
     <mergeCell ref="N61:Q61"/>
     <mergeCell ref="B57:C57"/>
     <mergeCell ref="D12:O12"/>
-    <mergeCell ref="B1:R1"/>
-    <mergeCell ref="B2:R2"/>
-    <mergeCell ref="B3:R3"/>
-    <mergeCell ref="B4:R4"/>
-    <mergeCell ref="B5:R5"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B4" r:id="rId1" xr:uid="{5EAE8D1D-5A31-4631-AC47-0FB40220C481}"/>

</xml_diff>

<commit_message>
Page setup for report improve
</commit_message>
<xml_diff>
--- a/sample/VAR-REPORT.xlsx
+++ b/sample/VAR-REPORT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Miks\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23B95D1F-41B9-4F95-8A84-1E9331AEC594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D34F0E4-1370-479C-BE49-2AB65C4244E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{39334F03-1232-460D-B301-DE63E4B3EB5C}"/>
   </bookViews>
@@ -82,9 +82,6 @@
     <t>Name</t>
   </si>
   <si>
-    <t>Attraction Code</t>
-  </si>
-  <si>
     <t>Philippines</t>
   </si>
   <si>
@@ -149,6 +146,10 @@
   </si>
   <si>
     <t>City Tourism Officer CGDH-1</t>
+  </si>
+  <si>
+    <t>Attraction 
+Code</t>
   </si>
 </sst>
 </file>
@@ -1045,6 +1046,114 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -1083,114 +1192,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -1588,107 +1589,107 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:18" ht="15">
-      <c r="B1" s="68" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
-      <c r="E1" s="68"/>
-      <c r="F1" s="68"/>
-      <c r="G1" s="68"/>
-      <c r="H1" s="68"/>
-      <c r="I1" s="68"/>
-      <c r="J1" s="68"/>
-      <c r="K1" s="68"/>
-      <c r="L1" s="68"/>
-      <c r="M1" s="68"/>
-      <c r="N1" s="68"/>
-      <c r="O1" s="68"/>
-      <c r="P1" s="68"/>
-      <c r="Q1" s="68"/>
-      <c r="R1" s="68"/>
+      <c r="B1" s="59" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
+      <c r="I1" s="59"/>
+      <c r="J1" s="59"/>
+      <c r="K1" s="59"/>
+      <c r="L1" s="59"/>
+      <c r="M1" s="59"/>
+      <c r="N1" s="59"/>
+      <c r="O1" s="59"/>
+      <c r="P1" s="59"/>
+      <c r="Q1" s="59"/>
+      <c r="R1" s="59"/>
     </row>
     <row r="2" spans="2:18" ht="15">
-      <c r="B2" s="68" t="s">
+      <c r="B2" s="59" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="68"/>
-      <c r="D2" s="68"/>
-      <c r="E2" s="68"/>
-      <c r="F2" s="68"/>
-      <c r="G2" s="68"/>
-      <c r="H2" s="68"/>
-      <c r="I2" s="68"/>
-      <c r="J2" s="68"/>
-      <c r="K2" s="68"/>
-      <c r="L2" s="68"/>
-      <c r="M2" s="68"/>
-      <c r="N2" s="68"/>
-      <c r="O2" s="68"/>
-      <c r="P2" s="68"/>
-      <c r="Q2" s="68"/>
-      <c r="R2" s="68"/>
+      <c r="C2" s="59"/>
+      <c r="D2" s="59"/>
+      <c r="E2" s="59"/>
+      <c r="F2" s="59"/>
+      <c r="G2" s="59"/>
+      <c r="H2" s="59"/>
+      <c r="I2" s="59"/>
+      <c r="J2" s="59"/>
+      <c r="K2" s="59"/>
+      <c r="L2" s="59"/>
+      <c r="M2" s="59"/>
+      <c r="N2" s="59"/>
+      <c r="O2" s="59"/>
+      <c r="P2" s="59"/>
+      <c r="Q2" s="59"/>
+      <c r="R2" s="59"/>
     </row>
     <row r="3" spans="2:18">
-      <c r="B3" s="69" t="s">
+      <c r="B3" s="60" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="69"/>
-      <c r="D3" s="69"/>
-      <c r="E3" s="69"/>
-      <c r="F3" s="69"/>
-      <c r="G3" s="69"/>
-      <c r="H3" s="69"/>
-      <c r="I3" s="69"/>
-      <c r="J3" s="69"/>
-      <c r="K3" s="69"/>
-      <c r="L3" s="69"/>
-      <c r="M3" s="69"/>
-      <c r="N3" s="69"/>
-      <c r="O3" s="69"/>
-      <c r="P3" s="69"/>
-      <c r="Q3" s="69"/>
-      <c r="R3" s="69"/>
+      <c r="C3" s="60"/>
+      <c r="D3" s="60"/>
+      <c r="E3" s="60"/>
+      <c r="F3" s="60"/>
+      <c r="G3" s="60"/>
+      <c r="H3" s="60"/>
+      <c r="I3" s="60"/>
+      <c r="J3" s="60"/>
+      <c r="K3" s="60"/>
+      <c r="L3" s="60"/>
+      <c r="M3" s="60"/>
+      <c r="N3" s="60"/>
+      <c r="O3" s="60"/>
+      <c r="P3" s="60"/>
+      <c r="Q3" s="60"/>
+      <c r="R3" s="60"/>
     </row>
     <row r="4" spans="2:18">
-      <c r="B4" s="70" t="s">
+      <c r="B4" s="61" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="70"/>
-      <c r="D4" s="70"/>
-      <c r="E4" s="70"/>
-      <c r="F4" s="70"/>
-      <c r="G4" s="70"/>
-      <c r="H4" s="70"/>
-      <c r="I4" s="70"/>
-      <c r="J4" s="70"/>
-      <c r="K4" s="70"/>
-      <c r="L4" s="70"/>
-      <c r="M4" s="70"/>
-      <c r="N4" s="70"/>
-      <c r="O4" s="70"/>
-      <c r="P4" s="70"/>
-      <c r="Q4" s="70"/>
-      <c r="R4" s="70"/>
+      <c r="C4" s="61"/>
+      <c r="D4" s="61"/>
+      <c r="E4" s="61"/>
+      <c r="F4" s="61"/>
+      <c r="G4" s="61"/>
+      <c r="H4" s="61"/>
+      <c r="I4" s="61"/>
+      <c r="J4" s="61"/>
+      <c r="K4" s="61"/>
+      <c r="L4" s="61"/>
+      <c r="M4" s="61"/>
+      <c r="N4" s="61"/>
+      <c r="O4" s="61"/>
+      <c r="P4" s="61"/>
+      <c r="Q4" s="61"/>
+      <c r="R4" s="61"/>
     </row>
     <row r="5" spans="2:18" ht="15">
-      <c r="B5" s="71"/>
-      <c r="C5" s="71"/>
-      <c r="D5" s="71"/>
-      <c r="E5" s="71"/>
-      <c r="F5" s="71"/>
-      <c r="G5" s="71"/>
-      <c r="H5" s="71"/>
-      <c r="I5" s="71"/>
-      <c r="J5" s="71"/>
-      <c r="K5" s="71"/>
-      <c r="L5" s="71"/>
-      <c r="M5" s="71"/>
-      <c r="N5" s="71"/>
-      <c r="O5" s="71"/>
-      <c r="P5" s="71"/>
-      <c r="Q5" s="71"/>
-      <c r="R5" s="71"/>
+      <c r="B5" s="62"/>
+      <c r="C5" s="62"/>
+      <c r="D5" s="62"/>
+      <c r="E5" s="62"/>
+      <c r="F5" s="62"/>
+      <c r="G5" s="62"/>
+      <c r="H5" s="62"/>
+      <c r="I5" s="62"/>
+      <c r="J5" s="62"/>
+      <c r="K5" s="62"/>
+      <c r="L5" s="62"/>
+      <c r="M5" s="62"/>
+      <c r="N5" s="62"/>
+      <c r="O5" s="62"/>
+      <c r="P5" s="62"/>
+      <c r="Q5" s="62"/>
+      <c r="R5" s="62"/>
     </row>
     <row r="6" spans="2:18" ht="15">
       <c r="B6" s="2" t="s">
@@ -1710,7 +1711,7 @@
       <c r="P6" s="3"/>
       <c r="Q6" s="3"/>
       <c r="R6" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="2:18" ht="14.25" customHeight="1">
@@ -1817,129 +1818,129 @@
       <c r="R11" s="9"/>
     </row>
     <row r="12" spans="2:18" ht="16.5" customHeight="1">
-      <c r="B12" s="92" t="s">
+      <c r="B12" s="83" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="93"/>
-      <c r="D12" s="64" t="s">
+      <c r="C12" s="84"/>
+      <c r="D12" s="92" t="s">
         <v>10</v>
       </c>
-      <c r="E12" s="65"/>
-      <c r="F12" s="65"/>
-      <c r="G12" s="65"/>
-      <c r="H12" s="65"/>
-      <c r="I12" s="65"/>
-      <c r="J12" s="65"/>
-      <c r="K12" s="65"/>
-      <c r="L12" s="65"/>
-      <c r="M12" s="65"/>
-      <c r="N12" s="65"/>
-      <c r="O12" s="66"/>
-      <c r="P12" s="82" t="s">
+      <c r="E12" s="93"/>
+      <c r="F12" s="93"/>
+      <c r="G12" s="93"/>
+      <c r="H12" s="93"/>
+      <c r="I12" s="93"/>
+      <c r="J12" s="93"/>
+      <c r="K12" s="93"/>
+      <c r="L12" s="93"/>
+      <c r="M12" s="93"/>
+      <c r="N12" s="93"/>
+      <c r="O12" s="94"/>
+      <c r="P12" s="73" t="s">
         <v>11</v>
       </c>
-      <c r="Q12" s="83"/>
-      <c r="R12" s="84"/>
+      <c r="Q12" s="74"/>
+      <c r="R12" s="75"/>
     </row>
     <row r="13" spans="2:18" ht="15" customHeight="1">
-      <c r="B13" s="72" t="s">
+      <c r="B13" s="63" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="75" t="s">
+      <c r="C13" s="66" t="s">
+        <v>35</v>
+      </c>
+      <c r="D13" s="78" t="s">
         <v>13</v>
       </c>
-      <c r="D13" s="87" t="s">
+      <c r="E13" s="79"/>
+      <c r="F13" s="79"/>
+      <c r="G13" s="79"/>
+      <c r="H13" s="79"/>
+      <c r="I13" s="79"/>
+      <c r="J13" s="79"/>
+      <c r="K13" s="79"/>
+      <c r="L13" s="79"/>
+      <c r="M13" s="63" t="s">
         <v>14</v>
       </c>
-      <c r="E13" s="88"/>
-      <c r="F13" s="88"/>
-      <c r="G13" s="88"/>
-      <c r="H13" s="88"/>
-      <c r="I13" s="88"/>
-      <c r="J13" s="88"/>
-      <c r="K13" s="88"/>
-      <c r="L13" s="88"/>
-      <c r="M13" s="72" t="s">
+      <c r="N13" s="69"/>
+      <c r="O13" s="70"/>
+      <c r="P13" s="64"/>
+      <c r="Q13" s="76"/>
+      <c r="R13" s="77"/>
+    </row>
+    <row r="14" spans="2:18" ht="28.5" customHeight="1" thickBot="1">
+      <c r="B14" s="64"/>
+      <c r="C14" s="67"/>
+      <c r="D14" s="80" t="s">
+        <v>25</v>
+      </c>
+      <c r="E14" s="81"/>
+      <c r="F14" s="82"/>
+      <c r="G14" s="80" t="s">
+        <v>26</v>
+      </c>
+      <c r="H14" s="81"/>
+      <c r="I14" s="82"/>
+      <c r="J14" s="80" t="s">
+        <v>27</v>
+      </c>
+      <c r="K14" s="81"/>
+      <c r="L14" s="82"/>
+      <c r="M14" s="65"/>
+      <c r="N14" s="71"/>
+      <c r="O14" s="72"/>
+      <c r="P14" s="65"/>
+      <c r="Q14" s="71"/>
+      <c r="R14" s="72"/>
+    </row>
+    <row r="15" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
+      <c r="B15" s="65"/>
+      <c r="C15" s="68"/>
+      <c r="D15" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="N13" s="78"/>
-      <c r="O13" s="79"/>
-      <c r="P13" s="73"/>
-      <c r="Q13" s="85"/>
-      <c r="R13" s="86"/>
-    </row>
-    <row r="14" spans="2:18" ht="28.5" customHeight="1" thickBot="1">
-      <c r="B14" s="73"/>
-      <c r="C14" s="76"/>
-      <c r="D14" s="89" t="s">
-        <v>26</v>
-      </c>
-      <c r="E14" s="90"/>
-      <c r="F14" s="91"/>
-      <c r="G14" s="89" t="s">
-        <v>27</v>
-      </c>
-      <c r="H14" s="90"/>
-      <c r="I14" s="91"/>
-      <c r="J14" s="89" t="s">
-        <v>28</v>
-      </c>
-      <c r="K14" s="90"/>
-      <c r="L14" s="91"/>
-      <c r="M14" s="74"/>
-      <c r="N14" s="80"/>
-      <c r="O14" s="81"/>
-      <c r="P14" s="74"/>
-      <c r="Q14" s="80"/>
-      <c r="R14" s="81"/>
-    </row>
-    <row r="15" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
-      <c r="B15" s="74"/>
-      <c r="C15" s="77"/>
-      <c r="D15" s="10" t="s">
+      <c r="E15" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="E15" s="11" t="s">
+      <c r="F15" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="F15" s="12" t="s">
+      <c r="G15" s="55" t="s">
+        <v>15</v>
+      </c>
+      <c r="H15" s="55" t="s">
+        <v>16</v>
+      </c>
+      <c r="I15" s="55" t="s">
+        <v>17</v>
+      </c>
+      <c r="J15" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="K15" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="L15" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="M15" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="G15" s="55" t="s">
+      <c r="N15" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="H15" s="55" t="s">
+      <c r="O15" s="45" t="s">
         <v>17</v>
       </c>
-      <c r="I15" s="55" t="s">
-        <v>18</v>
-      </c>
-      <c r="J15" s="10" t="s">
+      <c r="P15" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q15" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="K15" s="13" t="s">
+      <c r="R15" s="12" t="s">
         <v>17</v>
-      </c>
-      <c r="L15" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="M15" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="N15" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="O15" s="45" t="s">
-        <v>18</v>
-      </c>
-      <c r="P15" s="12" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q15" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="R15" s="12" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="16" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
@@ -3583,10 +3584,10 @@
       </c>
     </row>
     <row r="57" spans="2:18" ht="33.75" customHeight="1" thickBot="1">
-      <c r="B57" s="62" t="s">
-        <v>20</v>
-      </c>
-      <c r="C57" s="63"/>
+      <c r="B57" s="90" t="s">
+        <v>19</v>
+      </c>
+      <c r="C57" s="91"/>
       <c r="D57" s="41">
         <f>SUM(D16:D56)</f>
         <v>0</v>
@@ -3650,7 +3651,7 @@
     </row>
     <row r="58" spans="2:18" ht="15.75" customHeight="1">
       <c r="B58" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
@@ -3671,64 +3672,64 @@
     </row>
     <row r="59" spans="2:18" ht="15.75" customHeight="1">
       <c r="B59" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F59" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F59" s="1" t="s">
+      <c r="N59" s="85" t="s">
         <v>23</v>
       </c>
-      <c r="N59" s="57" t="s">
-        <v>24</v>
-      </c>
-      <c r="O59" s="57"/>
+      <c r="O59" s="85"/>
     </row>
     <row r="60" spans="2:18" ht="21" customHeight="1"/>
     <row r="61" spans="2:18" ht="21" customHeight="1">
       <c r="B61" s="56" t="s">
+        <v>31</v>
+      </c>
+      <c r="G61" s="86" t="s">
         <v>32</v>
       </c>
-      <c r="G61" s="58" t="s">
+      <c r="H61" s="87"/>
+      <c r="I61" s="87"/>
+      <c r="J61" s="87"/>
+      <c r="N61" s="88" t="s">
         <v>33</v>
       </c>
-      <c r="H61" s="59"/>
-      <c r="I61" s="59"/>
-      <c r="J61" s="59"/>
-      <c r="N61" s="60" t="s">
-        <v>34</v>
-      </c>
-      <c r="O61" s="61"/>
-      <c r="P61" s="61"/>
-      <c r="Q61" s="61"/>
+      <c r="O61" s="89"/>
+      <c r="P61" s="89"/>
+      <c r="Q61" s="89"/>
     </row>
     <row r="62" spans="2:18" ht="21" customHeight="1">
       <c r="B62" s="43" t="s">
+        <v>28</v>
+      </c>
+      <c r="G62" s="58" t="s">
         <v>29</v>
       </c>
-      <c r="G62" s="67" t="s">
-        <v>30</v>
-      </c>
-      <c r="H62" s="67"/>
-      <c r="I62" s="67"/>
-      <c r="J62" s="67"/>
-      <c r="N62" s="67" t="s">
-        <v>35</v>
-      </c>
-      <c r="O62" s="67"/>
-      <c r="P62" s="67"/>
-      <c r="Q62" s="67"/>
+      <c r="H62" s="58"/>
+      <c r="I62" s="58"/>
+      <c r="J62" s="58"/>
+      <c r="N62" s="58" t="s">
+        <v>34</v>
+      </c>
+      <c r="O62" s="58"/>
+      <c r="P62" s="58"/>
+      <c r="Q62" s="58"/>
     </row>
     <row r="63" spans="2:18" ht="21" customHeight="1">
-      <c r="G63" s="67"/>
-      <c r="H63" s="67"/>
-      <c r="I63" s="67"/>
-      <c r="J63" s="67"/>
-      <c r="N63" s="94"/>
-      <c r="O63" s="94"/>
-      <c r="P63" s="94"/>
-      <c r="Q63" s="94"/>
+      <c r="G63" s="58"/>
+      <c r="H63" s="58"/>
+      <c r="I63" s="58"/>
+      <c r="J63" s="58"/>
+      <c r="N63" s="57"/>
+      <c r="O63" s="57"/>
+      <c r="P63" s="57"/>
+      <c r="Q63" s="57"/>
     </row>
     <row r="64" spans="2:18" ht="21" customHeight="1">
       <c r="B64" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="65" spans="2:2" ht="21" customHeight="1">
@@ -3757,6 +3758,11 @@
     <row r="86" ht="21" customHeight="1"/>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="N59:O59"/>
+    <mergeCell ref="G61:J61"/>
+    <mergeCell ref="N61:Q61"/>
+    <mergeCell ref="B57:C57"/>
+    <mergeCell ref="D12:O12"/>
     <mergeCell ref="N62:Q62"/>
     <mergeCell ref="G62:J63"/>
     <mergeCell ref="B1:R1"/>
@@ -3773,11 +3779,6 @@
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="J14:L14"/>
     <mergeCell ref="G14:I14"/>
-    <mergeCell ref="N59:O59"/>
-    <mergeCell ref="G61:J61"/>
-    <mergeCell ref="N61:Q61"/>
-    <mergeCell ref="B57:C57"/>
-    <mergeCell ref="D12:O12"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B4" r:id="rId1" xr:uid="{5EAE8D1D-5A31-4631-AC47-0FB40220C481}"/>

</xml_diff>

<commit_message>
VAR2 report format fixed and updated to latest version
</commit_message>
<xml_diff>
--- a/sample/VAR-REPORT.xlsx
+++ b/sample/VAR-REPORT.xlsx
@@ -5,10 +5,10 @@
   <workbookPr showInkAnnotation="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Miks\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Miks\Desktop\MIKO\flutter\e-turismo\e-turismo-backend\sample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D34F0E4-1370-479C-BE49-2AB65C4244E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA227311-DB9A-477E-9BC7-3FC08BD04C43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{39334F03-1232-460D-B301-DE63E4B3EB5C}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="VAR 2M LGU Month Report" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'VAR 2M LGU Month Report'!$A$1:$R$64</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'VAR 2M LGU Month Report'!$A$1:$R$71</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,19 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="36">
-  <si>
-    <t>Republic of the Philippines</t>
-  </si>
-  <si>
-    <t>City Government of San Pablo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Information Center, Doña Leonila Park, City Hall Compound, San Pablo City </t>
-  </si>
-  <si>
-    <t>e-mail:  tourism.sanpablo@yahoo.com      Tel./Fax No.:  (049)562-1429</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="37">
   <si>
     <t xml:space="preserve">Tourism Attraction Visitor Record </t>
   </si>
@@ -151,12 +139,27 @@
     <t>Attraction 
 Code</t>
   </si>
+  <si>
+    <t xml:space="preserve">                                              Republic of the Philippines</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                                         City Government of San Pablo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                             Tourism Information Center, Doña Leonila Park</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                                        City Hall Compound, San Pablo City  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">            OFFICE OF CITY TOURISM</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="ＭＳ Ｐゴシック"/>
@@ -240,6 +243,18 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -838,7 +853,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="95">
+  <cellXfs count="113">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0"/>
@@ -1054,17 +1069,49 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1154,45 +1201,42 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="41" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1217,22 +1261,22 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>1038225</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:colOff>2106705</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>100853</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>2085975</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>104775</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>669737</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>11667</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1116" name="Picture 1">
+        <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F9185117-5518-39A1-9783-ABB9EE87868A}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FFE6212A-A5DB-4D53-B07E-9BC678CF81BA}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1241,7 +1285,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -1255,8 +1299,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="1143000" y="57150"/>
-          <a:ext cx="1047750" cy="609600"/>
+          <a:off x="2207558" y="481853"/>
+          <a:ext cx="1330885" cy="818490"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1282,6 +1326,67 @@
               <a:headEnd/>
               <a:tailEnd/>
             </a14:hiddenLine>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>68035</xdr:colOff>
+      <xdr:row>67</xdr:row>
+      <xdr:rowOff>244929</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>2009054</xdr:colOff>
+      <xdr:row>69</xdr:row>
+      <xdr:rowOff>262410</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9C128632-4E60-47D5-8990-8987B33FEF0C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="176892" y="14056179"/>
+          <a:ext cx="1941019" cy="561767"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
           </a:ext>
         </a:extLst>
       </xdr:spPr>
@@ -1578,8 +1683,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06E5140E-548F-489B-AF45-015A55956581}">
-  <dimension ref="B1:R86"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <dimension ref="B1:R93"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="1.375" style="1" customWidth="1"/>
     <col min="2" max="2" width="36.375" style="1" customWidth="1"/>
@@ -1588,644 +1693,512 @@
     <col min="19" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:18" ht="15">
-      <c r="B1" s="59" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="59"/>
-      <c r="D1" s="59"/>
-      <c r="E1" s="59"/>
-      <c r="F1" s="59"/>
-      <c r="G1" s="59"/>
-      <c r="H1" s="59"/>
-      <c r="I1" s="59"/>
-      <c r="J1" s="59"/>
-      <c r="K1" s="59"/>
-      <c r="L1" s="59"/>
-      <c r="M1" s="59"/>
-      <c r="N1" s="59"/>
-      <c r="O1" s="59"/>
-      <c r="P1" s="59"/>
-      <c r="Q1" s="59"/>
-      <c r="R1" s="59"/>
-    </row>
-    <row r="2" spans="2:18" ht="15">
-      <c r="B2" s="59" t="s">
+    <row r="1" spans="2:18" ht="15" x14ac:dyDescent="0.2">
+      <c r="B1" s="94"/>
+      <c r="C1" s="94"/>
+      <c r="D1" s="94"/>
+      <c r="E1" s="94"/>
+      <c r="F1" s="94"/>
+      <c r="G1" s="94"/>
+      <c r="H1" s="94"/>
+      <c r="I1" s="94"/>
+      <c r="J1" s="94"/>
+      <c r="K1" s="94"/>
+      <c r="L1" s="94"/>
+      <c r="M1" s="94"/>
+      <c r="N1" s="94"/>
+      <c r="O1" s="94"/>
+      <c r="P1" s="94"/>
+      <c r="Q1" s="94"/>
+      <c r="R1" s="94"/>
+    </row>
+    <row r="2" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="94"/>
+      <c r="C2" s="94"/>
+      <c r="D2" s="94"/>
+      <c r="E2" s="94"/>
+      <c r="F2" s="94"/>
+      <c r="G2" s="94"/>
+      <c r="H2" s="94"/>
+      <c r="I2" s="94"/>
+      <c r="J2" s="94"/>
+      <c r="K2" s="94"/>
+      <c r="L2" s="94"/>
+      <c r="M2" s="94"/>
+      <c r="N2" s="94"/>
+      <c r="O2" s="94"/>
+      <c r="P2" s="94"/>
+      <c r="Q2" s="94"/>
+      <c r="R2" s="94"/>
+    </row>
+    <row r="3" spans="2:18" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="B3" s="95"/>
+      <c r="C3" s="96"/>
+      <c r="D3" s="96"/>
+      <c r="E3" s="96"/>
+      <c r="F3" s="92" t="s">
+        <v>32</v>
+      </c>
+      <c r="G3" s="92"/>
+      <c r="H3" s="92"/>
+      <c r="I3" s="92"/>
+      <c r="J3" s="92"/>
+      <c r="K3" s="92"/>
+      <c r="L3" s="92"/>
+      <c r="M3" s="92"/>
+      <c r="N3" s="92"/>
+      <c r="O3" s="92"/>
+      <c r="P3" s="92"/>
+      <c r="Q3" s="92"/>
+      <c r="R3" s="93"/>
+    </row>
+    <row r="4" spans="2:18" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="B4" s="97"/>
+      <c r="C4" s="98"/>
+      <c r="D4" s="98"/>
+      <c r="E4" s="98"/>
+      <c r="F4" s="110" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4" s="110"/>
+      <c r="H4" s="110"/>
+      <c r="I4" s="110"/>
+      <c r="J4" s="110"/>
+      <c r="K4" s="110"/>
+      <c r="L4" s="110"/>
+      <c r="M4" s="110"/>
+      <c r="N4" s="110"/>
+      <c r="O4" s="110"/>
+      <c r="P4" s="110"/>
+      <c r="Q4" s="110"/>
+      <c r="R4" s="107"/>
+    </row>
+    <row r="5" spans="2:18" ht="15" x14ac:dyDescent="0.25">
+      <c r="B5" s="99"/>
+      <c r="C5" s="100"/>
+      <c r="D5" s="100"/>
+      <c r="E5" s="100"/>
+      <c r="F5" s="111" t="s">
+        <v>34</v>
+      </c>
+      <c r="G5" s="111"/>
+      <c r="H5" s="111"/>
+      <c r="I5" s="111"/>
+      <c r="J5" s="111"/>
+      <c r="K5" s="111"/>
+      <c r="L5" s="111"/>
+      <c r="M5" s="111"/>
+      <c r="N5" s="111"/>
+      <c r="O5" s="111"/>
+      <c r="P5" s="111"/>
+      <c r="Q5" s="111"/>
+      <c r="R5" s="108"/>
+    </row>
+    <row r="6" spans="2:18" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="B6" s="101"/>
+      <c r="C6" s="102"/>
+      <c r="D6" s="102"/>
+      <c r="E6" s="102"/>
+      <c r="F6" s="111" t="s">
+        <v>35</v>
+      </c>
+      <c r="G6" s="111"/>
+      <c r="H6" s="111"/>
+      <c r="I6" s="111"/>
+      <c r="J6" s="111"/>
+      <c r="K6" s="111"/>
+      <c r="L6" s="111"/>
+      <c r="M6" s="111"/>
+      <c r="N6" s="111"/>
+      <c r="O6" s="111"/>
+      <c r="P6" s="111"/>
+      <c r="Q6" s="111"/>
+      <c r="R6" s="108"/>
+    </row>
+    <row r="7" spans="2:18" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B7" s="101"/>
+      <c r="C7" s="102"/>
+      <c r="D7" s="102"/>
+      <c r="E7" s="102"/>
+      <c r="F7" s="102"/>
+      <c r="G7" s="102"/>
+      <c r="H7" s="102"/>
+      <c r="I7" s="102"/>
+      <c r="J7" s="102"/>
+      <c r="K7" s="102"/>
+      <c r="L7" s="102"/>
+      <c r="M7" s="102"/>
+      <c r="N7" s="102"/>
+      <c r="O7" s="102"/>
+      <c r="P7" s="102"/>
+      <c r="Q7" s="102"/>
+      <c r="R7" s="103"/>
+    </row>
+    <row r="8" spans="2:18" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="104"/>
+      <c r="C8" s="105"/>
+      <c r="D8" s="105"/>
+      <c r="E8" s="105"/>
+      <c r="F8" s="105"/>
+      <c r="G8" s="105"/>
+      <c r="H8" s="112" t="s">
+        <v>36</v>
+      </c>
+      <c r="I8" s="112"/>
+      <c r="J8" s="112"/>
+      <c r="K8" s="112"/>
+      <c r="L8" s="112"/>
+      <c r="M8" s="112"/>
+      <c r="N8" s="105"/>
+      <c r="O8" s="105"/>
+      <c r="P8" s="105"/>
+      <c r="Q8" s="105"/>
+      <c r="R8" s="106"/>
+    </row>
+    <row r="9" spans="2:18" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H9" s="109"/>
+      <c r="I9" s="109"/>
+      <c r="J9" s="109"/>
+      <c r="K9" s="109"/>
+      <c r="L9" s="109"/>
+      <c r="M9" s="109"/>
+    </row>
+    <row r="10" spans="2:18" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="11" spans="2:18" ht="15" x14ac:dyDescent="0.25">
+      <c r="B11" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C11" s="2"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
+      <c r="J11" s="3"/>
+      <c r="K11" s="3"/>
+      <c r="L11" s="3"/>
+      <c r="M11" s="3"/>
+      <c r="N11" s="3"/>
+      <c r="O11" s="3"/>
+      <c r="P11" s="3"/>
+      <c r="Q11" s="3"/>
+      <c r="R11" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="2:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B12" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="59"/>
-      <c r="D2" s="59"/>
-      <c r="E2" s="59"/>
-      <c r="F2" s="59"/>
-      <c r="G2" s="59"/>
-      <c r="H2" s="59"/>
-      <c r="I2" s="59"/>
-      <c r="J2" s="59"/>
-      <c r="K2" s="59"/>
-      <c r="L2" s="59"/>
-      <c r="M2" s="59"/>
-      <c r="N2" s="59"/>
-      <c r="O2" s="59"/>
-      <c r="P2" s="59"/>
-      <c r="Q2" s="59"/>
-      <c r="R2" s="59"/>
-    </row>
-    <row r="3" spans="2:18">
-      <c r="B3" s="60" t="s">
+      <c r="C12" s="4"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
+      <c r="J12" s="3"/>
+      <c r="K12" s="3"/>
+      <c r="L12" s="3"/>
+      <c r="M12" s="3"/>
+      <c r="N12" s="3"/>
+      <c r="O12" s="3"/>
+      <c r="P12" s="3"/>
+      <c r="Q12" s="3"/>
+      <c r="R12" s="3"/>
+    </row>
+    <row r="13" spans="2:18" ht="8.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
+      <c r="J13" s="3"/>
+      <c r="K13" s="3"/>
+      <c r="L13" s="3"/>
+      <c r="M13" s="3"/>
+      <c r="N13" s="3"/>
+      <c r="O13" s="3"/>
+      <c r="P13" s="3"/>
+      <c r="Q13" s="3"/>
+      <c r="R13" s="3"/>
+    </row>
+    <row r="14" spans="2:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="60"/>
-      <c r="D3" s="60"/>
-      <c r="E3" s="60"/>
-      <c r="F3" s="60"/>
-      <c r="G3" s="60"/>
-      <c r="H3" s="60"/>
-      <c r="I3" s="60"/>
-      <c r="J3" s="60"/>
-      <c r="K3" s="60"/>
-      <c r="L3" s="60"/>
-      <c r="M3" s="60"/>
-      <c r="N3" s="60"/>
-      <c r="O3" s="60"/>
-      <c r="P3" s="60"/>
-      <c r="Q3" s="60"/>
-      <c r="R3" s="60"/>
-    </row>
-    <row r="4" spans="2:18">
-      <c r="B4" s="61" t="s">
+      <c r="F14" s="5"/>
+      <c r="G14" s="6"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="7"/>
+      <c r="K14" s="7"/>
+      <c r="L14" s="7"/>
+      <c r="M14" s="7"/>
+      <c r="N14" s="7"/>
+      <c r="O14" s="7"/>
+      <c r="P14" s="7"/>
+      <c r="Q14" s="7"/>
+      <c r="R14" s="44"/>
+    </row>
+    <row r="15" spans="2:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="61"/>
-      <c r="D4" s="61"/>
-      <c r="E4" s="61"/>
-      <c r="F4" s="61"/>
-      <c r="G4" s="61"/>
-      <c r="H4" s="61"/>
-      <c r="I4" s="61"/>
-      <c r="J4" s="61"/>
-      <c r="K4" s="61"/>
-      <c r="L4" s="61"/>
-      <c r="M4" s="61"/>
-      <c r="N4" s="61"/>
-      <c r="O4" s="61"/>
-      <c r="P4" s="61"/>
-      <c r="Q4" s="61"/>
-      <c r="R4" s="61"/>
-    </row>
-    <row r="5" spans="2:18" ht="15">
-      <c r="B5" s="62"/>
-      <c r="C5" s="62"/>
-      <c r="D5" s="62"/>
-      <c r="E5" s="62"/>
-      <c r="F5" s="62"/>
-      <c r="G5" s="62"/>
-      <c r="H5" s="62"/>
-      <c r="I5" s="62"/>
-      <c r="J5" s="62"/>
-      <c r="K5" s="62"/>
-      <c r="L5" s="62"/>
-      <c r="M5" s="62"/>
-      <c r="N5" s="62"/>
-      <c r="O5" s="62"/>
-      <c r="P5" s="62"/>
-      <c r="Q5" s="62"/>
-      <c r="R5" s="62"/>
-    </row>
-    <row r="6" spans="2:18" ht="15">
-      <c r="B6" s="2" t="s">
+      <c r="F15" s="5"/>
+      <c r="G15" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="2"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
-      <c r="K6" s="3"/>
-      <c r="L6" s="3"/>
-      <c r="M6" s="3"/>
-      <c r="N6" s="3"/>
-      <c r="O6" s="3"/>
-      <c r="P6" s="3"/>
-      <c r="Q6" s="3"/>
-      <c r="R6" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="2:18" ht="14.25" customHeight="1">
-      <c r="B7" s="4" t="s">
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
+      <c r="J15" s="8"/>
+      <c r="K15" s="8"/>
+      <c r="L15" s="8"/>
+      <c r="M15" s="8"/>
+      <c r="N15" s="8"/>
+      <c r="O15" s="8"/>
+      <c r="P15" s="8"/>
+      <c r="Q15" s="8"/>
+      <c r="R15" s="44"/>
+    </row>
+    <row r="16" spans="2:18" ht="8.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="9"/>
+      <c r="I16" s="9"/>
+      <c r="J16" s="9"/>
+      <c r="K16" s="9"/>
+      <c r="L16" s="9"/>
+      <c r="M16" s="44"/>
+      <c r="N16" s="44"/>
+      <c r="O16" s="44"/>
+      <c r="P16" s="9"/>
+      <c r="Q16" s="9"/>
+      <c r="R16" s="9"/>
+    </row>
+    <row r="17" spans="2:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="90" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3"/>
-      <c r="L7" s="3"/>
-      <c r="M7" s="3"/>
-      <c r="N7" s="3"/>
-      <c r="O7" s="3"/>
-      <c r="P7" s="3"/>
-      <c r="Q7" s="3"/>
-      <c r="R7" s="3"/>
-    </row>
-    <row r="8" spans="2:18" ht="8.25" customHeight="1">
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-      <c r="L8" s="3"/>
-      <c r="M8" s="3"/>
-      <c r="N8" s="3"/>
-      <c r="O8" s="3"/>
-      <c r="P8" s="3"/>
-      <c r="Q8" s="3"/>
-      <c r="R8" s="3"/>
-    </row>
-    <row r="9" spans="2:18" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="5" t="s">
+      <c r="C17" s="91"/>
+      <c r="D17" s="66" t="s">
         <v>6</v>
       </c>
-      <c r="F9" s="5"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="7"/>
-      <c r="J9" s="7"/>
-      <c r="K9" s="7"/>
-      <c r="L9" s="7"/>
-      <c r="M9" s="7"/>
-      <c r="N9" s="7"/>
-      <c r="O9" s="7"/>
-      <c r="P9" s="7"/>
-      <c r="Q9" s="7"/>
-      <c r="R9" s="44"/>
-    </row>
-    <row r="10" spans="2:18" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="5" t="s">
+      <c r="E17" s="67"/>
+      <c r="F17" s="67"/>
+      <c r="G17" s="67"/>
+      <c r="H17" s="67"/>
+      <c r="I17" s="67"/>
+      <c r="J17" s="67"/>
+      <c r="K17" s="67"/>
+      <c r="L17" s="67"/>
+      <c r="M17" s="67"/>
+      <c r="N17" s="67"/>
+      <c r="O17" s="68"/>
+      <c r="P17" s="80" t="s">
         <v>7</v>
       </c>
-      <c r="F10" s="5"/>
-      <c r="G10" s="8" t="s">
+      <c r="Q17" s="81"/>
+      <c r="R17" s="82"/>
+    </row>
+    <row r="18" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B18" s="70" t="s">
         <v>8</v>
       </c>
-      <c r="H10" s="8"/>
-      <c r="I10" s="8"/>
-      <c r="J10" s="8"/>
-      <c r="K10" s="8"/>
-      <c r="L10" s="8"/>
-      <c r="M10" s="8"/>
-      <c r="N10" s="8"/>
-      <c r="O10" s="8"/>
-      <c r="P10" s="8"/>
-      <c r="Q10" s="8"/>
-      <c r="R10" s="44"/>
-    </row>
-    <row r="11" spans="2:18" ht="8.25" customHeight="1" thickBot="1">
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
-      <c r="K11" s="9"/>
-      <c r="L11" s="9"/>
-      <c r="M11" s="44"/>
-      <c r="N11" s="44"/>
-      <c r="O11" s="44"/>
-      <c r="P11" s="9"/>
-      <c r="Q11" s="9"/>
-      <c r="R11" s="9"/>
-    </row>
-    <row r="12" spans="2:18" ht="16.5" customHeight="1">
-      <c r="B12" s="83" t="s">
+      <c r="C18" s="73" t="s">
+        <v>31</v>
+      </c>
+      <c r="D18" s="85" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="84"/>
-      <c r="D12" s="92" t="s">
+      <c r="E18" s="86"/>
+      <c r="F18" s="86"/>
+      <c r="G18" s="86"/>
+      <c r="H18" s="86"/>
+      <c r="I18" s="86"/>
+      <c r="J18" s="86"/>
+      <c r="K18" s="86"/>
+      <c r="L18" s="86"/>
+      <c r="M18" s="70" t="s">
         <v>10</v>
       </c>
-      <c r="E12" s="93"/>
-      <c r="F12" s="93"/>
-      <c r="G12" s="93"/>
-      <c r="H12" s="93"/>
-      <c r="I12" s="93"/>
-      <c r="J12" s="93"/>
-      <c r="K12" s="93"/>
-      <c r="L12" s="93"/>
-      <c r="M12" s="93"/>
-      <c r="N12" s="93"/>
-      <c r="O12" s="94"/>
-      <c r="P12" s="73" t="s">
+      <c r="N18" s="76"/>
+      <c r="O18" s="77"/>
+      <c r="P18" s="71"/>
+      <c r="Q18" s="83"/>
+      <c r="R18" s="84"/>
+    </row>
+    <row r="19" spans="2:18" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="71"/>
+      <c r="C19" s="74"/>
+      <c r="D19" s="87" t="s">
+        <v>21</v>
+      </c>
+      <c r="E19" s="88"/>
+      <c r="F19" s="89"/>
+      <c r="G19" s="87" t="s">
+        <v>22</v>
+      </c>
+      <c r="H19" s="88"/>
+      <c r="I19" s="89"/>
+      <c r="J19" s="87" t="s">
+        <v>23</v>
+      </c>
+      <c r="K19" s="88"/>
+      <c r="L19" s="89"/>
+      <c r="M19" s="72"/>
+      <c r="N19" s="78"/>
+      <c r="O19" s="79"/>
+      <c r="P19" s="72"/>
+      <c r="Q19" s="78"/>
+      <c r="R19" s="79"/>
+    </row>
+    <row r="20" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="72"/>
+      <c r="C20" s="75"/>
+      <c r="D20" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="Q12" s="74"/>
-      <c r="R12" s="75"/>
-    </row>
-    <row r="13" spans="2:18" ht="15" customHeight="1">
-      <c r="B13" s="63" t="s">
+      <c r="E20" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="66" t="s">
-        <v>35</v>
-      </c>
-      <c r="D13" s="78" t="s">
+      <c r="F20" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="E13" s="79"/>
-      <c r="F13" s="79"/>
-      <c r="G13" s="79"/>
-      <c r="H13" s="79"/>
-      <c r="I13" s="79"/>
-      <c r="J13" s="79"/>
-      <c r="K13" s="79"/>
-      <c r="L13" s="79"/>
-      <c r="M13" s="63" t="s">
+      <c r="G20" s="55" t="s">
+        <v>11</v>
+      </c>
+      <c r="H20" s="55" t="s">
+        <v>12</v>
+      </c>
+      <c r="I20" s="55" t="s">
+        <v>13</v>
+      </c>
+      <c r="J20" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="K20" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="L20" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="M20" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="N13" s="69"/>
-      <c r="O13" s="70"/>
-      <c r="P13" s="64"/>
-      <c r="Q13" s="76"/>
-      <c r="R13" s="77"/>
-    </row>
-    <row r="14" spans="2:18" ht="28.5" customHeight="1" thickBot="1">
-      <c r="B14" s="64"/>
-      <c r="C14" s="67"/>
-      <c r="D14" s="80" t="s">
-        <v>25</v>
-      </c>
-      <c r="E14" s="81"/>
-      <c r="F14" s="82"/>
-      <c r="G14" s="80" t="s">
-        <v>26</v>
-      </c>
-      <c r="H14" s="81"/>
-      <c r="I14" s="82"/>
-      <c r="J14" s="80" t="s">
-        <v>27</v>
-      </c>
-      <c r="K14" s="81"/>
-      <c r="L14" s="82"/>
-      <c r="M14" s="65"/>
-      <c r="N14" s="71"/>
-      <c r="O14" s="72"/>
-      <c r="P14" s="65"/>
-      <c r="Q14" s="71"/>
-      <c r="R14" s="72"/>
-    </row>
-    <row r="15" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
-      <c r="B15" s="65"/>
-      <c r="C15" s="68"/>
-      <c r="D15" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="E15" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="F15" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="G15" s="55" t="s">
-        <v>15</v>
-      </c>
-      <c r="H15" s="55" t="s">
-        <v>16</v>
-      </c>
-      <c r="I15" s="55" t="s">
-        <v>17</v>
-      </c>
-      <c r="J15" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="K15" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="L15" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="M15" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="N15" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="O15" s="45" t="s">
-        <v>17</v>
-      </c>
-      <c r="P15" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q15" s="12" t="s">
-        <v>16</v>
-      </c>
-      <c r="R15" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="16" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
-      <c r="B16" s="14"/>
-      <c r="C16" s="15"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="18">
-        <f t="shared" ref="F16:F45" si="0">D16+E16</f>
-        <v>0</v>
-      </c>
-      <c r="G16" s="19"/>
-      <c r="H16" s="47"/>
-      <c r="I16" s="48">
-        <f t="shared" ref="I16:I56" si="1">G16+H16</f>
-        <v>0</v>
-      </c>
-      <c r="J16" s="19"/>
-      <c r="K16" s="20"/>
-      <c r="L16" s="46">
-        <f t="shared" ref="L16:L45" si="2">J16+K16</f>
-        <v>0</v>
-      </c>
-      <c r="M16" s="19"/>
-      <c r="N16" s="47"/>
-      <c r="O16" s="48">
-        <f t="shared" ref="O16:O45" si="3">M16+N16</f>
-        <v>0</v>
-      </c>
-      <c r="P16" s="49">
-        <f>D16+G16+J16+M16</f>
-        <v>0</v>
-      </c>
-      <c r="Q16" s="49">
-        <f>E16+H16+K16+N16</f>
-        <v>0</v>
-      </c>
-      <c r="R16" s="49">
-        <f>F16+I16+L16+O16</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
-      <c r="B17" s="21"/>
-      <c r="C17" s="22"/>
-      <c r="D17" s="23"/>
-      <c r="E17" s="24"/>
-      <c r="F17" s="18">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G17" s="25"/>
-      <c r="H17" s="50"/>
-      <c r="I17" s="48">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J17" s="25"/>
-      <c r="K17" s="26"/>
-      <c r="L17" s="46">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="M17" s="25"/>
-      <c r="N17" s="50"/>
-      <c r="O17" s="48">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="P17" s="49">
-        <f t="shared" ref="P17:P56" si="4">D17+G17+J17+M17</f>
-        <v>0</v>
-      </c>
-      <c r="Q17" s="49">
-        <f t="shared" ref="Q17:Q56" si="5">E17+H17+K17+N17</f>
-        <v>0</v>
-      </c>
-      <c r="R17" s="49">
-        <f t="shared" ref="R17:R57" si="6">F17+I17+L17+O17</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
-      <c r="B18" s="21"/>
-      <c r="C18" s="22"/>
-      <c r="D18" s="23"/>
-      <c r="E18" s="24"/>
-      <c r="F18" s="18">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G18" s="25"/>
-      <c r="H18" s="50"/>
-      <c r="I18" s="48">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J18" s="25"/>
-      <c r="K18" s="26"/>
-      <c r="L18" s="46">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="M18" s="25"/>
-      <c r="N18" s="50"/>
-      <c r="O18" s="48">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="P18" s="49">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q18" s="49">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R18" s="49">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
-      <c r="B19" s="21"/>
-      <c r="C19" s="22"/>
-      <c r="D19" s="27"/>
-      <c r="E19" s="28"/>
-      <c r="F19" s="18">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G19" s="29"/>
-      <c r="H19" s="51"/>
-      <c r="I19" s="48">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J19" s="29"/>
-      <c r="K19" s="30"/>
-      <c r="L19" s="46">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="M19" s="29"/>
-      <c r="N19" s="51"/>
-      <c r="O19" s="48">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="P19" s="49">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q19" s="49">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R19" s="49">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
-      <c r="B20" s="21"/>
-      <c r="C20" s="22"/>
-      <c r="D20" s="27"/>
-      <c r="E20" s="28"/>
-      <c r="F20" s="18">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G20" s="29"/>
-      <c r="H20" s="51"/>
-      <c r="I20" s="48">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J20" s="29"/>
-      <c r="K20" s="30"/>
-      <c r="L20" s="46">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="M20" s="29"/>
-      <c r="N20" s="51"/>
-      <c r="O20" s="48">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="P20" s="49">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q20" s="49">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R20" s="49">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
-      <c r="B21" s="21"/>
-      <c r="C21" s="22"/>
-      <c r="D21" s="27"/>
-      <c r="E21" s="28"/>
+      <c r="N20" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="O20" s="45" t="s">
+        <v>13</v>
+      </c>
+      <c r="P20" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q20" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="R20" s="12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="21" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="14"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="17"/>
       <c r="F21" s="18">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G21" s="29"/>
-      <c r="H21" s="51"/>
+        <f t="shared" ref="F21:F50" si="0">D21+E21</f>
+        <v>0</v>
+      </c>
+      <c r="G21" s="19"/>
+      <c r="H21" s="47"/>
       <c r="I21" s="48">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J21" s="29"/>
-      <c r="K21" s="30"/>
+        <f t="shared" ref="I21:I61" si="1">G21+H21</f>
+        <v>0</v>
+      </c>
+      <c r="J21" s="19"/>
+      <c r="K21" s="20"/>
       <c r="L21" s="46">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="M21" s="29"/>
-      <c r="N21" s="51"/>
+        <f t="shared" ref="L21:L50" si="2">J21+K21</f>
+        <v>0</v>
+      </c>
+      <c r="M21" s="19"/>
+      <c r="N21" s="47"/>
       <c r="O21" s="48">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="O21:O50" si="3">M21+N21</f>
         <v>0</v>
       </c>
       <c r="P21" s="49">
-        <f t="shared" si="4"/>
+        <f>D21+G21+J21+M21</f>
         <v>0</v>
       </c>
       <c r="Q21" s="49">
-        <f t="shared" si="5"/>
+        <f>E21+H21+K21+N21</f>
         <v>0</v>
       </c>
       <c r="R21" s="49">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
+        <f>F21+I21+L21+O21</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B22" s="21"/>
       <c r="C22" s="22"/>
-      <c r="D22" s="27"/>
-      <c r="E22" s="28"/>
+      <c r="D22" s="23"/>
+      <c r="E22" s="24"/>
       <c r="F22" s="18">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G22" s="29"/>
-      <c r="H22" s="51"/>
+      <c r="G22" s="25"/>
+      <c r="H22" s="50"/>
       <c r="I22" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J22" s="29"/>
-      <c r="K22" s="30"/>
+      <c r="J22" s="25"/>
+      <c r="K22" s="26"/>
       <c r="L22" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M22" s="29"/>
-      <c r="N22" s="51"/>
+      <c r="M22" s="25"/>
+      <c r="N22" s="50"/>
       <c r="O22" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P22" s="49">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="P22:P61" si="4">D22+G22+J22+M22</f>
         <v>0</v>
       </c>
       <c r="Q22" s="49">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="Q22:Q61" si="5">E22+H22+K22+N22</f>
         <v>0</v>
       </c>
       <c r="R22" s="49">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
+        <f t="shared" ref="R22:R62" si="6">F22+I22+L22+O22</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B23" s="21"/>
-      <c r="C23" s="31"/>
+      <c r="C23" s="22"/>
       <c r="D23" s="23"/>
       <c r="E23" s="24"/>
       <c r="F23" s="18">
@@ -2263,9 +2236,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
+    <row r="24" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B24" s="21"/>
-      <c r="C24" s="31"/>
+      <c r="C24" s="22"/>
       <c r="D24" s="27"/>
       <c r="E24" s="28"/>
       <c r="F24" s="18">
@@ -2303,29 +2276,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
+    <row r="25" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B25" s="21"/>
-      <c r="C25" s="31"/>
-      <c r="D25" s="23"/>
-      <c r="E25" s="24"/>
+      <c r="C25" s="22"/>
+      <c r="D25" s="27"/>
+      <c r="E25" s="28"/>
       <c r="F25" s="18">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G25" s="25"/>
-      <c r="H25" s="50"/>
+      <c r="G25" s="29"/>
+      <c r="H25" s="51"/>
       <c r="I25" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J25" s="25"/>
-      <c r="K25" s="26"/>
+      <c r="J25" s="29"/>
+      <c r="K25" s="30"/>
       <c r="L25" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M25" s="25"/>
-      <c r="N25" s="50"/>
+      <c r="M25" s="29"/>
+      <c r="N25" s="51"/>
       <c r="O25" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -2343,9 +2316,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
+    <row r="26" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B26" s="21"/>
-      <c r="C26" s="31"/>
+      <c r="C26" s="22"/>
       <c r="D26" s="27"/>
       <c r="E26" s="28"/>
       <c r="F26" s="18">
@@ -2383,29 +2356,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
+    <row r="27" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B27" s="21"/>
-      <c r="C27" s="31"/>
-      <c r="D27" s="23"/>
-      <c r="E27" s="24"/>
+      <c r="C27" s="22"/>
+      <c r="D27" s="27"/>
+      <c r="E27" s="28"/>
       <c r="F27" s="18">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G27" s="25"/>
-      <c r="H27" s="50"/>
+      <c r="G27" s="29"/>
+      <c r="H27" s="51"/>
       <c r="I27" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J27" s="25"/>
-      <c r="K27" s="26"/>
+      <c r="J27" s="29"/>
+      <c r="K27" s="30"/>
       <c r="L27" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M27" s="25"/>
-      <c r="N27" s="50"/>
+      <c r="M27" s="29"/>
+      <c r="N27" s="51"/>
       <c r="O27" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -2423,29 +2396,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
+    <row r="28" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B28" s="21"/>
       <c r="C28" s="31"/>
-      <c r="D28" s="27"/>
-      <c r="E28" s="28"/>
+      <c r="D28" s="23"/>
+      <c r="E28" s="24"/>
       <c r="F28" s="18">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G28" s="29"/>
-      <c r="H28" s="51"/>
+      <c r="G28" s="25"/>
+      <c r="H28" s="50"/>
       <c r="I28" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J28" s="29"/>
-      <c r="K28" s="30"/>
+      <c r="J28" s="25"/>
+      <c r="K28" s="26"/>
       <c r="L28" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M28" s="29"/>
-      <c r="N28" s="51"/>
+      <c r="M28" s="25"/>
+      <c r="N28" s="50"/>
       <c r="O28" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -2463,29 +2436,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="2:18" ht="17.25" hidden="1" customHeight="1">
+    <row r="29" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B29" s="21"/>
       <c r="C29" s="31"/>
-      <c r="D29" s="32"/>
-      <c r="E29" s="33"/>
+      <c r="D29" s="27"/>
+      <c r="E29" s="28"/>
       <c r="F29" s="18">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G29" s="34"/>
-      <c r="H29" s="52"/>
+      <c r="G29" s="29"/>
+      <c r="H29" s="51"/>
       <c r="I29" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J29" s="34"/>
-      <c r="K29" s="35"/>
+      <c r="J29" s="29"/>
+      <c r="K29" s="30"/>
       <c r="L29" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M29" s="34"/>
-      <c r="N29" s="52"/>
+      <c r="M29" s="29"/>
+      <c r="N29" s="51"/>
       <c r="O29" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -2503,7 +2476,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
+    <row r="30" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B30" s="21"/>
       <c r="C30" s="31"/>
       <c r="D30" s="23"/>
@@ -2543,7 +2516,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
+    <row r="31" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B31" s="21"/>
       <c r="C31" s="31"/>
       <c r="D31" s="27"/>
@@ -2583,7 +2556,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
+    <row r="32" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B32" s="21"/>
       <c r="C32" s="31"/>
       <c r="D32" s="23"/>
@@ -2623,29 +2596,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
+    <row r="33" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B33" s="21"/>
       <c r="C33" s="31"/>
-      <c r="D33" s="23"/>
-      <c r="E33" s="24"/>
+      <c r="D33" s="27"/>
+      <c r="E33" s="28"/>
       <c r="F33" s="18">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G33" s="25"/>
-      <c r="H33" s="50"/>
+      <c r="G33" s="29"/>
+      <c r="H33" s="51"/>
       <c r="I33" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J33" s="25"/>
-      <c r="K33" s="26"/>
+      <c r="J33" s="29"/>
+      <c r="K33" s="30"/>
       <c r="L33" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M33" s="25"/>
-      <c r="N33" s="50"/>
+      <c r="M33" s="29"/>
+      <c r="N33" s="51"/>
       <c r="O33" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -2663,29 +2636,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
+    <row r="34" spans="2:18" ht="17.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B34" s="21"/>
       <c r="C34" s="31"/>
-      <c r="D34" s="27"/>
-      <c r="E34" s="28"/>
+      <c r="D34" s="32"/>
+      <c r="E34" s="33"/>
       <c r="F34" s="18">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G34" s="29"/>
-      <c r="H34" s="51"/>
+      <c r="G34" s="34"/>
+      <c r="H34" s="52"/>
       <c r="I34" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J34" s="29"/>
-      <c r="K34" s="30"/>
+      <c r="J34" s="34"/>
+      <c r="K34" s="35"/>
       <c r="L34" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M34" s="29"/>
-      <c r="N34" s="51"/>
+      <c r="M34" s="34"/>
+      <c r="N34" s="52"/>
       <c r="O34" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -2703,29 +2676,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
+    <row r="35" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B35" s="21"/>
       <c r="C35" s="31"/>
-      <c r="D35" s="27"/>
-      <c r="E35" s="28"/>
+      <c r="D35" s="23"/>
+      <c r="E35" s="24"/>
       <c r="F35" s="18">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G35" s="29"/>
-      <c r="H35" s="51"/>
+      <c r="G35" s="25"/>
+      <c r="H35" s="50"/>
       <c r="I35" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J35" s="29"/>
-      <c r="K35" s="30"/>
+      <c r="J35" s="25"/>
+      <c r="K35" s="26"/>
       <c r="L35" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M35" s="29"/>
-      <c r="N35" s="51"/>
+      <c r="M35" s="25"/>
+      <c r="N35" s="50"/>
       <c r="O35" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -2743,29 +2716,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="2:18" ht="17.25" hidden="1" customHeight="1">
+    <row r="36" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B36" s="21"/>
       <c r="C36" s="31"/>
-      <c r="D36" s="23"/>
-      <c r="E36" s="24"/>
+      <c r="D36" s="27"/>
+      <c r="E36" s="28"/>
       <c r="F36" s="18">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G36" s="25"/>
-      <c r="H36" s="50"/>
+      <c r="G36" s="29"/>
+      <c r="H36" s="51"/>
       <c r="I36" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J36" s="25"/>
-      <c r="K36" s="26"/>
+      <c r="J36" s="29"/>
+      <c r="K36" s="30"/>
       <c r="L36" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M36" s="25"/>
-      <c r="N36" s="50"/>
+      <c r="M36" s="29"/>
+      <c r="N36" s="51"/>
       <c r="O36" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -2783,7 +2756,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
+    <row r="37" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B37" s="21"/>
       <c r="C37" s="31"/>
       <c r="D37" s="23"/>
@@ -2823,29 +2796,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
-      <c r="B38" s="36"/>
+    <row r="38" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B38" s="21"/>
       <c r="C38" s="31"/>
-      <c r="D38" s="37"/>
-      <c r="E38" s="38"/>
+      <c r="D38" s="23"/>
+      <c r="E38" s="24"/>
       <c r="F38" s="18">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G38" s="37"/>
-      <c r="H38" s="38"/>
+      <c r="G38" s="25"/>
+      <c r="H38" s="50"/>
       <c r="I38" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J38" s="37"/>
-      <c r="K38" s="38"/>
+      <c r="J38" s="25"/>
+      <c r="K38" s="26"/>
       <c r="L38" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M38" s="37"/>
-      <c r="N38" s="38"/>
+      <c r="M38" s="25"/>
+      <c r="N38" s="50"/>
       <c r="O38" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -2863,29 +2836,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
-      <c r="B39" s="36"/>
+    <row r="39" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B39" s="21"/>
       <c r="C39" s="31"/>
-      <c r="D39" s="37"/>
-      <c r="E39" s="38"/>
+      <c r="D39" s="27"/>
+      <c r="E39" s="28"/>
       <c r="F39" s="18">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G39" s="37"/>
-      <c r="H39" s="38"/>
+      <c r="G39" s="29"/>
+      <c r="H39" s="51"/>
       <c r="I39" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J39" s="37"/>
-      <c r="K39" s="38"/>
+      <c r="J39" s="29"/>
+      <c r="K39" s="30"/>
       <c r="L39" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M39" s="37"/>
-      <c r="N39" s="38"/>
+      <c r="M39" s="29"/>
+      <c r="N39" s="51"/>
       <c r="O39" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -2903,29 +2876,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
-      <c r="B40" s="36"/>
+    <row r="40" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B40" s="21"/>
       <c r="C40" s="31"/>
-      <c r="D40" s="23"/>
-      <c r="E40" s="24"/>
+      <c r="D40" s="27"/>
+      <c r="E40" s="28"/>
       <c r="F40" s="18">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G40" s="25"/>
-      <c r="H40" s="50"/>
+      <c r="G40" s="29"/>
+      <c r="H40" s="51"/>
       <c r="I40" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J40" s="25"/>
-      <c r="K40" s="26"/>
+      <c r="J40" s="29"/>
+      <c r="K40" s="30"/>
       <c r="L40" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M40" s="25"/>
-      <c r="N40" s="50"/>
+      <c r="M40" s="29"/>
+      <c r="N40" s="51"/>
       <c r="O40" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -2943,8 +2916,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
-      <c r="B41" s="36"/>
+    <row r="41" spans="2:18" ht="17.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B41" s="21"/>
       <c r="C41" s="31"/>
       <c r="D41" s="23"/>
       <c r="E41" s="24"/>
@@ -2983,29 +2956,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
-      <c r="B42" s="36"/>
+    <row r="42" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B42" s="21"/>
       <c r="C42" s="31"/>
-      <c r="D42" s="37"/>
-      <c r="E42" s="38"/>
+      <c r="D42" s="23"/>
+      <c r="E42" s="24"/>
       <c r="F42" s="18">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G42" s="37"/>
-      <c r="H42" s="38"/>
+      <c r="G42" s="25"/>
+      <c r="H42" s="50"/>
       <c r="I42" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J42" s="37"/>
-      <c r="K42" s="38"/>
+      <c r="J42" s="25"/>
+      <c r="K42" s="26"/>
       <c r="L42" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M42" s="37"/>
-      <c r="N42" s="38"/>
+      <c r="M42" s="25"/>
+      <c r="N42" s="50"/>
       <c r="O42" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -3023,7 +2996,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
+    <row r="43" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B43" s="36"/>
       <c r="C43" s="31"/>
       <c r="D43" s="37"/>
@@ -3063,29 +3036,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="2:18" ht="17.25" hidden="1" customHeight="1">
+    <row r="44" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B44" s="36"/>
       <c r="C44" s="31"/>
-      <c r="D44" s="32"/>
-      <c r="E44" s="33"/>
+      <c r="D44" s="37"/>
+      <c r="E44" s="38"/>
       <c r="F44" s="18">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G44" s="34"/>
-      <c r="H44" s="52"/>
+      <c r="G44" s="37"/>
+      <c r="H44" s="38"/>
       <c r="I44" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J44" s="34"/>
-      <c r="K44" s="35"/>
+      <c r="J44" s="37"/>
+      <c r="K44" s="38"/>
       <c r="L44" s="46">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M44" s="34"/>
-      <c r="N44" s="52"/>
+      <c r="M44" s="37"/>
+      <c r="N44" s="38"/>
       <c r="O44" s="48">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -3103,7 +3076,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
+    <row r="45" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B45" s="36"/>
       <c r="C45" s="31"/>
       <c r="D45" s="23"/>
@@ -3143,13 +3116,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
+    <row r="46" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B46" s="36"/>
       <c r="C46" s="31"/>
       <c r="D46" s="23"/>
       <c r="E46" s="24"/>
       <c r="F46" s="18">
-        <f t="shared" ref="F46:F56" si="7">D46+E46</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="G46" s="25"/>
@@ -3161,13 +3134,13 @@
       <c r="J46" s="25"/>
       <c r="K46" s="26"/>
       <c r="L46" s="46">
-        <f t="shared" ref="L46:L56" si="8">J46+K46</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M46" s="25"/>
       <c r="N46" s="50"/>
       <c r="O46" s="48">
-        <f t="shared" ref="O46:O56" si="9">M46+N46</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P46" s="49">
@@ -3183,31 +3156,31 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
+    <row r="47" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B47" s="36"/>
       <c r="C47" s="31"/>
-      <c r="D47" s="23"/>
-      <c r="E47" s="24"/>
+      <c r="D47" s="37"/>
+      <c r="E47" s="38"/>
       <c r="F47" s="18">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="G47" s="25"/>
-      <c r="H47" s="50"/>
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G47" s="37"/>
+      <c r="H47" s="38"/>
       <c r="I47" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J47" s="25"/>
-      <c r="K47" s="26"/>
+      <c r="J47" s="37"/>
+      <c r="K47" s="38"/>
       <c r="L47" s="46">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="M47" s="25"/>
-      <c r="N47" s="50"/>
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="M47" s="37"/>
+      <c r="N47" s="38"/>
       <c r="O47" s="48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P47" s="49">
@@ -3223,31 +3196,31 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
+    <row r="48" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B48" s="36"/>
       <c r="C48" s="31"/>
-      <c r="D48" s="23"/>
-      <c r="E48" s="24"/>
+      <c r="D48" s="37"/>
+      <c r="E48" s="38"/>
       <c r="F48" s="18">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="G48" s="25"/>
-      <c r="H48" s="50"/>
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G48" s="37"/>
+      <c r="H48" s="38"/>
       <c r="I48" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J48" s="25"/>
-      <c r="K48" s="26"/>
+      <c r="J48" s="37"/>
+      <c r="K48" s="38"/>
       <c r="L48" s="46">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="M48" s="25"/>
-      <c r="N48" s="50"/>
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="M48" s="37"/>
+      <c r="N48" s="38"/>
       <c r="O48" s="48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P48" s="49">
@@ -3263,31 +3236,31 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
+    <row r="49" spans="2:18" ht="17.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B49" s="36"/>
       <c r="C49" s="31"/>
-      <c r="D49" s="37"/>
-      <c r="E49" s="38"/>
+      <c r="D49" s="32"/>
+      <c r="E49" s="33"/>
       <c r="F49" s="18">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="G49" s="37"/>
-      <c r="H49" s="38"/>
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G49" s="34"/>
+      <c r="H49" s="52"/>
       <c r="I49" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J49" s="37"/>
-      <c r="K49" s="38"/>
+      <c r="J49" s="34"/>
+      <c r="K49" s="35"/>
       <c r="L49" s="46">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="M49" s="37"/>
-      <c r="N49" s="38"/>
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="M49" s="34"/>
+      <c r="N49" s="52"/>
       <c r="O49" s="48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P49" s="49">
@@ -3303,13 +3276,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
+    <row r="50" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B50" s="36"/>
       <c r="C50" s="31"/>
       <c r="D50" s="23"/>
       <c r="E50" s="24"/>
       <c r="F50" s="18">
-        <f t="shared" si="7"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="G50" s="25"/>
@@ -3321,13 +3294,13 @@
       <c r="J50" s="25"/>
       <c r="K50" s="26"/>
       <c r="L50" s="46">
-        <f t="shared" si="8"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M50" s="25"/>
       <c r="N50" s="50"/>
       <c r="O50" s="48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P50" s="49">
@@ -3343,31 +3316,31 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
+    <row r="51" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B51" s="36"/>
       <c r="C51" s="31"/>
-      <c r="D51" s="37"/>
-      <c r="E51" s="38"/>
+      <c r="D51" s="23"/>
+      <c r="E51" s="24"/>
       <c r="F51" s="18">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="G51" s="37"/>
-      <c r="H51" s="38"/>
+        <f t="shared" ref="F51:F61" si="7">D51+E51</f>
+        <v>0</v>
+      </c>
+      <c r="G51" s="25"/>
+      <c r="H51" s="50"/>
       <c r="I51" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J51" s="37"/>
-      <c r="K51" s="38"/>
+      <c r="J51" s="25"/>
+      <c r="K51" s="26"/>
       <c r="L51" s="46">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="M51" s="37"/>
-      <c r="N51" s="38"/>
+        <f t="shared" ref="L51:L61" si="8">J51+K51</f>
+        <v>0</v>
+      </c>
+      <c r="M51" s="25"/>
+      <c r="N51" s="50"/>
       <c r="O51" s="48">
-        <f t="shared" si="9"/>
+        <f t="shared" ref="O51:O61" si="9">M51+N51</f>
         <v>0</v>
       </c>
       <c r="P51" s="49">
@@ -3383,29 +3356,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
+    <row r="52" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B52" s="36"/>
       <c r="C52" s="31"/>
-      <c r="D52" s="37"/>
-      <c r="E52" s="38"/>
+      <c r="D52" s="23"/>
+      <c r="E52" s="24"/>
       <c r="F52" s="18">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="G52" s="37"/>
-      <c r="H52" s="38"/>
+      <c r="G52" s="25"/>
+      <c r="H52" s="50"/>
       <c r="I52" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J52" s="37"/>
-      <c r="K52" s="38"/>
+      <c r="J52" s="25"/>
+      <c r="K52" s="26"/>
       <c r="L52" s="46">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="M52" s="37"/>
-      <c r="N52" s="38"/>
+      <c r="M52" s="25"/>
+      <c r="N52" s="50"/>
       <c r="O52" s="48">
         <f t="shared" si="9"/>
         <v>0</v>
@@ -3423,7 +3396,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
+    <row r="53" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B53" s="36"/>
       <c r="C53" s="31"/>
       <c r="D53" s="23"/>
@@ -3463,29 +3436,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
+    <row r="54" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B54" s="36"/>
       <c r="C54" s="31"/>
-      <c r="D54" s="23"/>
-      <c r="E54" s="24"/>
+      <c r="D54" s="37"/>
+      <c r="E54" s="38"/>
       <c r="F54" s="18">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="G54" s="25"/>
-      <c r="H54" s="50"/>
+      <c r="G54" s="37"/>
+      <c r="H54" s="38"/>
       <c r="I54" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J54" s="25"/>
-      <c r="K54" s="26"/>
+      <c r="J54" s="37"/>
+      <c r="K54" s="38"/>
       <c r="L54" s="46">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="M54" s="25"/>
-      <c r="N54" s="50"/>
+      <c r="M54" s="37"/>
+      <c r="N54" s="38"/>
       <c r="O54" s="48">
         <f t="shared" si="9"/>
         <v>0</v>
@@ -3503,7 +3476,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
+    <row r="55" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B55" s="36"/>
       <c r="C55" s="31"/>
       <c r="D55" s="23"/>
@@ -3543,9 +3516,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="2:18" ht="17.25" customHeight="1" thickBot="1">
-      <c r="B56" s="39"/>
-      <c r="C56" s="40"/>
+    <row r="56" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B56" s="36"/>
+      <c r="C56" s="31"/>
       <c r="D56" s="37"/>
       <c r="E56" s="38"/>
       <c r="F56" s="18">
@@ -3583,65 +3556,39 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="2:18" ht="33.75" customHeight="1" thickBot="1">
-      <c r="B57" s="90" t="s">
-        <v>19</v>
-      </c>
-      <c r="C57" s="91"/>
-      <c r="D57" s="41">
-        <f>SUM(D16:D56)</f>
-        <v>0</v>
-      </c>
-      <c r="E57" s="41">
-        <f>SUM(E16:E56)</f>
-        <v>0</v>
-      </c>
-      <c r="F57" s="42">
-        <f t="shared" ref="F57:Q57" si="10">SUM(F16:F56)</f>
-        <v>0</v>
-      </c>
-      <c r="G57" s="41">
-        <f>SUM(G16:G56)</f>
-        <v>0</v>
-      </c>
-      <c r="H57" s="41">
-        <f>SUM(H16:H56)</f>
-        <v>0</v>
-      </c>
-      <c r="I57" s="42">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="J57" s="41">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="K57" s="41">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="L57" s="41">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="M57" s="41">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="N57" s="41">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="O57" s="41">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="P57" s="53">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="Q57" s="42">
-        <f t="shared" si="10"/>
+    <row r="57" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B57" s="36"/>
+      <c r="C57" s="31"/>
+      <c r="D57" s="37"/>
+      <c r="E57" s="38"/>
+      <c r="F57" s="18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="G57" s="37"/>
+      <c r="H57" s="38"/>
+      <c r="I57" s="48">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J57" s="37"/>
+      <c r="K57" s="38"/>
+      <c r="L57" s="46">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="M57" s="37"/>
+      <c r="N57" s="38"/>
+      <c r="O57" s="48">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="P57" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q57" s="49">
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="R57" s="49">
@@ -3649,144 +3596,387 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="2:18" ht="15.75" customHeight="1">
-      <c r="B58" s="4" t="s">
+    <row r="58" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B58" s="36"/>
+      <c r="C58" s="31"/>
+      <c r="D58" s="23"/>
+      <c r="E58" s="24"/>
+      <c r="F58" s="18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="G58" s="25"/>
+      <c r="H58" s="50"/>
+      <c r="I58" s="48">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J58" s="25"/>
+      <c r="K58" s="26"/>
+      <c r="L58" s="46">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="M58" s="25"/>
+      <c r="N58" s="50"/>
+      <c r="O58" s="48">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="P58" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q58" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R58" s="49">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B59" s="36"/>
+      <c r="C59" s="31"/>
+      <c r="D59" s="23"/>
+      <c r="E59" s="24"/>
+      <c r="F59" s="18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="G59" s="25"/>
+      <c r="H59" s="50"/>
+      <c r="I59" s="48">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J59" s="25"/>
+      <c r="K59" s="26"/>
+      <c r="L59" s="46">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="M59" s="25"/>
+      <c r="N59" s="50"/>
+      <c r="O59" s="48">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="P59" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q59" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R59" s="49">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B60" s="36"/>
+      <c r="C60" s="31"/>
+      <c r="D60" s="23"/>
+      <c r="E60" s="24"/>
+      <c r="F60" s="18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="G60" s="25"/>
+      <c r="H60" s="50"/>
+      <c r="I60" s="48">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J60" s="25"/>
+      <c r="K60" s="26"/>
+      <c r="L60" s="46">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="M60" s="25"/>
+      <c r="N60" s="50"/>
+      <c r="O60" s="48">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="P60" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q60" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R60" s="49">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="2:18" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B61" s="39"/>
+      <c r="C61" s="40"/>
+      <c r="D61" s="37"/>
+      <c r="E61" s="38"/>
+      <c r="F61" s="18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="G61" s="37"/>
+      <c r="H61" s="38"/>
+      <c r="I61" s="48">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J61" s="37"/>
+      <c r="K61" s="38"/>
+      <c r="L61" s="46">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="M61" s="37"/>
+      <c r="N61" s="38"/>
+      <c r="O61" s="48">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="P61" s="49">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q61" s="49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R61" s="49">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="2:18" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B62" s="64" t="s">
+        <v>15</v>
+      </c>
+      <c r="C62" s="65"/>
+      <c r="D62" s="41">
+        <f>SUM(D21:D61)</f>
+        <v>0</v>
+      </c>
+      <c r="E62" s="41">
+        <f>SUM(E21:E61)</f>
+        <v>0</v>
+      </c>
+      <c r="F62" s="42">
+        <f t="shared" ref="F62:Q62" si="10">SUM(F21:F61)</f>
+        <v>0</v>
+      </c>
+      <c r="G62" s="41">
+        <f>SUM(G21:G61)</f>
+        <v>0</v>
+      </c>
+      <c r="H62" s="41">
+        <f>SUM(H21:H61)</f>
+        <v>0</v>
+      </c>
+      <c r="I62" s="42">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J62" s="41">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="K62" s="41">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="L62" s="41">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="M62" s="41">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="N62" s="41">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="O62" s="41">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="P62" s="53">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="Q62" s="42">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="R62" s="49">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B63" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C63" s="4"/>
+      <c r="D63" s="4"/>
+      <c r="E63" s="4"/>
+      <c r="F63" s="4"/>
+      <c r="G63" s="4"/>
+      <c r="H63" s="4"/>
+      <c r="I63" s="4"/>
+      <c r="J63" s="4"/>
+      <c r="K63" s="4"/>
+      <c r="L63" s="4"/>
+      <c r="M63" s="4"/>
+      <c r="N63" s="4"/>
+      <c r="O63" s="4"/>
+      <c r="P63" s="4"/>
+      <c r="Q63" s="4"/>
+      <c r="R63" s="4"/>
+    </row>
+    <row r="64" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B64" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F64" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="N64" s="59" t="s">
+        <v>19</v>
+      </c>
+      <c r="O64" s="59"/>
+    </row>
+    <row r="65" spans="2:17" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="66" spans="2:17" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B66" s="56" t="s">
+        <v>27</v>
+      </c>
+      <c r="G66" s="60" t="s">
+        <v>28</v>
+      </c>
+      <c r="H66" s="61"/>
+      <c r="I66" s="61"/>
+      <c r="J66" s="61"/>
+      <c r="N66" s="62" t="s">
+        <v>29</v>
+      </c>
+      <c r="O66" s="63"/>
+      <c r="P66" s="63"/>
+      <c r="Q66" s="63"/>
+    </row>
+    <row r="67" spans="2:17" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B67" s="43" t="s">
+        <v>24</v>
+      </c>
+      <c r="G67" s="69" t="s">
+        <v>25</v>
+      </c>
+      <c r="H67" s="69"/>
+      <c r="I67" s="69"/>
+      <c r="J67" s="69"/>
+      <c r="N67" s="69" t="s">
+        <v>30</v>
+      </c>
+      <c r="O67" s="69"/>
+      <c r="P67" s="69"/>
+      <c r="Q67" s="69"/>
+    </row>
+    <row r="68" spans="2:17" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G68" s="69"/>
+      <c r="H68" s="69"/>
+      <c r="I68" s="69"/>
+      <c r="J68" s="69"/>
+      <c r="N68" s="57"/>
+      <c r="O68" s="57"/>
+      <c r="P68" s="57"/>
+      <c r="Q68" s="57"/>
+    </row>
+    <row r="69" spans="2:17" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G69" s="58"/>
+      <c r="H69" s="58"/>
+      <c r="I69" s="58"/>
+      <c r="J69" s="58"/>
+      <c r="N69" s="57"/>
+      <c r="O69" s="57"/>
+      <c r="P69" s="57"/>
+      <c r="Q69" s="57"/>
+    </row>
+    <row r="70" spans="2:17" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G70" s="58"/>
+      <c r="H70" s="58"/>
+      <c r="I70" s="58"/>
+      <c r="J70" s="58"/>
+      <c r="N70" s="57"/>
+      <c r="O70" s="57"/>
+      <c r="P70" s="57"/>
+      <c r="Q70" s="57"/>
+    </row>
+    <row r="71" spans="2:17" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B71" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C58" s="4"/>
-      <c r="D58" s="4"/>
-      <c r="E58" s="4"/>
-      <c r="F58" s="4"/>
-      <c r="G58" s="4"/>
-      <c r="H58" s="4"/>
-      <c r="I58" s="4"/>
-      <c r="J58" s="4"/>
-      <c r="K58" s="4"/>
-      <c r="L58" s="4"/>
-      <c r="M58" s="4"/>
-      <c r="N58" s="4"/>
-      <c r="O58" s="4"/>
-      <c r="P58" s="4"/>
-      <c r="Q58" s="4"/>
-      <c r="R58" s="4"/>
-    </row>
-    <row r="59" spans="2:18" ht="15.75" customHeight="1">
-      <c r="B59" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F59" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="N59" s="85" t="s">
-        <v>23</v>
-      </c>
-      <c r="O59" s="85"/>
-    </row>
-    <row r="60" spans="2:18" ht="21" customHeight="1"/>
-    <row r="61" spans="2:18" ht="21" customHeight="1">
-      <c r="B61" s="56" t="s">
-        <v>31</v>
-      </c>
-      <c r="G61" s="86" t="s">
-        <v>32</v>
-      </c>
-      <c r="H61" s="87"/>
-      <c r="I61" s="87"/>
-      <c r="J61" s="87"/>
-      <c r="N61" s="88" t="s">
-        <v>33</v>
-      </c>
-      <c r="O61" s="89"/>
-      <c r="P61" s="89"/>
-      <c r="Q61" s="89"/>
-    </row>
-    <row r="62" spans="2:18" ht="21" customHeight="1">
-      <c r="B62" s="43" t="s">
-        <v>28</v>
-      </c>
-      <c r="G62" s="58" t="s">
-        <v>29</v>
-      </c>
-      <c r="H62" s="58"/>
-      <c r="I62" s="58"/>
-      <c r="J62" s="58"/>
-      <c r="N62" s="58" t="s">
-        <v>34</v>
-      </c>
-      <c r="O62" s="58"/>
-      <c r="P62" s="58"/>
-      <c r="Q62" s="58"/>
-    </row>
-    <row r="63" spans="2:18" ht="21" customHeight="1">
-      <c r="G63" s="58"/>
-      <c r="H63" s="58"/>
-      <c r="I63" s="58"/>
-      <c r="J63" s="58"/>
-      <c r="N63" s="57"/>
-      <c r="O63" s="57"/>
-      <c r="P63" s="57"/>
-      <c r="Q63" s="57"/>
-    </row>
-    <row r="64" spans="2:18" ht="21" customHeight="1">
-      <c r="B64" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="65" spans="2:2" ht="21" customHeight="1">
-      <c r="B65" s="54"/>
-    </row>
-    <row r="66" spans="2:2" ht="21" customHeight="1"/>
-    <row r="67" spans="2:2" ht="21" customHeight="1"/>
-    <row r="68" spans="2:2" ht="21" customHeight="1"/>
-    <row r="69" spans="2:2" ht="21" customHeight="1"/>
-    <row r="70" spans="2:2" ht="21" customHeight="1"/>
-    <row r="71" spans="2:2" ht="21" customHeight="1"/>
-    <row r="72" spans="2:2" ht="21" customHeight="1"/>
-    <row r="73" spans="2:2" ht="21" customHeight="1"/>
-    <row r="74" spans="2:2" ht="21" customHeight="1"/>
-    <row r="75" spans="2:2" ht="21" customHeight="1"/>
-    <row r="76" spans="2:2" ht="21" customHeight="1"/>
-    <row r="77" spans="2:2" ht="21" customHeight="1"/>
-    <row r="78" spans="2:2" ht="21" customHeight="1"/>
-    <row r="79" spans="2:2" ht="21" customHeight="1"/>
-    <row r="80" spans="2:2" ht="21" customHeight="1"/>
-    <row r="81" ht="21" customHeight="1"/>
-    <row r="82" ht="21" customHeight="1"/>
-    <row r="83" ht="21" customHeight="1"/>
-    <row r="84" ht="21" customHeight="1"/>
-    <row r="85" ht="21" customHeight="1"/>
-    <row r="86" ht="21" customHeight="1"/>
+    </row>
+    <row r="72" spans="2:17" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B72" s="54"/>
+    </row>
+    <row r="73" spans="2:17" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="74" spans="2:17" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="75" spans="2:17" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="76" spans="2:17" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="77" spans="2:17" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="78" spans="2:17" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="79" spans="2:17" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="80" spans="2:17" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="81" s="1" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="82" s="1" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="83" s="1" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="84" s="1" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="85" s="1" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="86" s="1" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="87" s="1" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="88" s="1" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="89" s="1" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="90" s="1" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="91" s="1" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="92" s="1" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="93" s="1" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="N59:O59"/>
-    <mergeCell ref="G61:J61"/>
-    <mergeCell ref="N61:Q61"/>
-    <mergeCell ref="B57:C57"/>
-    <mergeCell ref="D12:O12"/>
-    <mergeCell ref="N62:Q62"/>
-    <mergeCell ref="G62:J63"/>
-    <mergeCell ref="B1:R1"/>
-    <mergeCell ref="B2:R2"/>
-    <mergeCell ref="B3:R3"/>
-    <mergeCell ref="B4:R4"/>
-    <mergeCell ref="B5:R5"/>
-    <mergeCell ref="B13:B15"/>
-    <mergeCell ref="C13:C15"/>
-    <mergeCell ref="M13:O14"/>
-    <mergeCell ref="P12:R14"/>
-    <mergeCell ref="D13:L13"/>
-    <mergeCell ref="D14:F14"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="J14:L14"/>
-    <mergeCell ref="G14:I14"/>
+    <mergeCell ref="H8:M8"/>
+    <mergeCell ref="F3:R3"/>
+    <mergeCell ref="F4:R4"/>
+    <mergeCell ref="F5:R5"/>
+    <mergeCell ref="F6:R6"/>
+    <mergeCell ref="N67:Q67"/>
+    <mergeCell ref="G67:J68"/>
+    <mergeCell ref="B18:B20"/>
+    <mergeCell ref="C18:C20"/>
+    <mergeCell ref="M18:O19"/>
+    <mergeCell ref="P17:R19"/>
+    <mergeCell ref="D18:L18"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="N64:O64"/>
+    <mergeCell ref="G66:J66"/>
+    <mergeCell ref="N66:Q66"/>
+    <mergeCell ref="B62:C62"/>
+    <mergeCell ref="D17:O17"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink ref="B4" r:id="rId1" xr:uid="{5EAE8D1D-5A31-4631-AC47-0FB40220C481}"/>
-  </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.78699912510936132" right="0.15699912510936134" top="0.11799978127734033" bottom="0.19599956255468068" header="0.15699912510936134" footer="0.15699912510936134"/>
-  <pageSetup paperSize="9" scale="58" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId2"/>
+  <pageSetup paperSize="9" scale="54" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
-  <drawing r:id="rId3"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>